<commit_message>
chore(evidencia-iso): Log operational evidence 16/10/2026 (REL-2026-107..110 & SUP-2026-1215 Veeam v13.1 / ReadyNAS / Smart City)
</commit_message>
<xml_diff>
--- a/SGC-AIMS-REG-001_MATRIZ_RIESGOS_Y_EVIDENCIA_OPERATIVA_90_DIAS.xlsx
+++ b/SGC-AIMS-REG-001_MATRIZ_RIESGOS_Y_EVIDENCIA_OPERATIVA_90_DIAS.xlsx
@@ -826,7 +826,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H8"/>
+  <dimension ref="A1:H12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -1140,6 +1140,174 @@
         </is>
       </c>
     </row>
+    <row r="9" ht="30" customHeight="1">
+      <c r="A9" s="3" t="inlineStr">
+        <is>
+          <t>REL-2026-107</t>
+        </is>
+      </c>
+      <c r="B9" s="4" t="inlineStr">
+        <is>
+          <t>15/10/2026</t>
+        </is>
+      </c>
+      <c r="C9" s="4" t="inlineStr">
+        <is>
+          <t>Infraestructura ThinkConnect — ReadyNAS Btrfs &amp; Veeam v13.1</t>
+        </is>
+      </c>
+      <c r="D9" s="4" t="inlineStr">
+        <is>
+          <t>Continuidad de Negocio (ISO 9001 Cl. 8.5)</t>
+        </is>
+      </c>
+      <c r="E9" s="4" t="inlineStr">
+        <is>
+          <t>Modernización a ReadyNAS OS 6.9.5 (5.44 TB Btrfs) y upgrade a Veeam Agent v13.1.1.700 en Server_IA y Notebook con réplicas secundarias.</t>
+        </is>
+      </c>
+      <c r="F9" s="4" t="inlineStr">
+        <is>
+          <t>Verificación de snapshots Btrfs anti-ransomware y sincronización de archivos .vbk.</t>
+        </is>
+      </c>
+      <c r="G9" s="4" t="inlineStr">
+        <is>
+          <t>Sincronizado en GEMINI.md</t>
+        </is>
+      </c>
+      <c r="H9" s="5" t="inlineStr">
+        <is>
+          <t>APROBADO</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="30" customHeight="1">
+      <c r="A10" s="6" t="inlineStr">
+        <is>
+          <t>REL-2026-108</t>
+        </is>
+      </c>
+      <c r="B10" s="7" t="inlineStr">
+        <is>
+          <t>16/10/2026</t>
+        </is>
+      </c>
+      <c r="C10" s="7" t="inlineStr">
+        <is>
+          <t>Proyecto 16 — Trilogía LATAM Smart City Awards 2027</t>
+        </is>
+      </c>
+      <c r="D10" s="7" t="inlineStr">
+        <is>
+          <t>Hito GovTech Internacional (ISO 42001)</t>
+        </is>
+      </c>
+      <c r="E10" s="7" t="inlineStr">
+        <is>
+          <t>Ratificación oficial de Fira Barcelona International admitiendo UrbanAgent OS (6acb97d97db00), TerraVolt DePIN (6acb8f3b47daa) y EcoCívica DePIN (6ad0e54955bc5).</t>
+        </is>
+      </c>
+      <c r="F10" s="7" t="inlineStr">
+        <is>
+          <t>Confirmación oficial de Secretaría Técnica (Paula Juyol) en plataforma Helice.</t>
+        </is>
+      </c>
+      <c r="G10" s="7" t="inlineStr">
+        <is>
+          <t>Sincronizado en Z:\Documentacion\16_...</t>
+        </is>
+      </c>
+      <c r="H10" s="5" t="inlineStr">
+        <is>
+          <t>APROBADO</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="30" customHeight="1">
+      <c r="A11" s="3" t="inlineStr">
+        <is>
+          <t>REL-2026-109</t>
+        </is>
+      </c>
+      <c r="B11" s="4" t="inlineStr">
+        <is>
+          <t>16/10/2026</t>
+        </is>
+      </c>
+      <c r="C11" s="4" t="inlineStr">
+        <is>
+          <t>Infraestructura — ThinkConnect IT Sentinel Companion</t>
+        </is>
+      </c>
+      <c r="D11" s="4" t="inlineStr">
+        <is>
+          <t>Monitoreo Automatizado 24/7 (SI)</t>
+        </is>
+      </c>
+      <c r="E11" s="4" t="inlineStr">
+        <is>
+          <t>Integración del método auditar_readynas() al motor de diagnóstico diario en Server_IA y reporte matutino por Gateway WAHA.</t>
+        </is>
+      </c>
+      <c r="F11" s="4" t="inlineStr">
+        <is>
+          <t>Ejecución en vivo (0.4s) validando capacidad Btrfs (5.41 TB libres) y réplicas Veeam.</t>
+        </is>
+      </c>
+      <c r="G11" s="4" t="inlineStr">
+        <is>
+          <t>Sincronizado en Server_IA</t>
+        </is>
+      </c>
+      <c r="H11" s="5" t="inlineStr">
+        <is>
+          <t>APROBADO</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="30" customHeight="1">
+      <c r="A12" s="6" t="inlineStr">
+        <is>
+          <t>REL-2026-110</t>
+        </is>
+      </c>
+      <c r="B12" s="7" t="inlineStr">
+        <is>
+          <t>16/10/2026</t>
+        </is>
+      </c>
+      <c r="C12" s="7" t="inlineStr">
+        <is>
+          <t>Proyecto 5 — EstudioConta Pro (Reel RIMI v4)</t>
+        </is>
+      </c>
+      <c r="D12" s="7" t="inlineStr">
+        <is>
+          <t>Mejora Continua y Control de Calidad Audio/Video</t>
+        </is>
+      </c>
+      <c r="E12" s="7" t="inlineStr">
+        <is>
+          <t>Re-masterización de Reel RIMI (Ley 27.802) con locución argentina es-AR-TomasNeural y filtro broadcast loudnorm (-16 LUFS).</t>
+        </is>
+      </c>
+      <c r="F12" s="7" t="inlineStr">
+        <is>
+          <t>Despliegue SFTP en VPS 1 y publicación verificada vía Graph API en Instagram.</t>
+        </is>
+      </c>
+      <c r="G12" s="7" t="inlineStr">
+        <is>
+          <t>Sincronizado en Z:\Documentacion\5_...</t>
+        </is>
+      </c>
+      <c r="H12" s="5" t="inlineStr">
+        <is>
+          <t>APROBADO</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:H1"/>
@@ -1154,7 +1322,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H5"/>
+  <dimension ref="A1:H6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -1337,6 +1505,48 @@
         </is>
       </c>
       <c r="H5" s="5" t="inlineStr">
+        <is>
+          <t>CERRADO CONFORME</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="30" customHeight="1">
+      <c r="A6" s="6" t="inlineStr">
+        <is>
+          <t>SUP-2026-1215</t>
+        </is>
+      </c>
+      <c r="B6" s="7" t="inlineStr">
+        <is>
+          <t>16/10/2026</t>
+        </is>
+      </c>
+      <c r="C6" s="7" t="inlineStr">
+        <is>
+          <t>Hormimac S.A.</t>
+        </is>
+      </c>
+      <c r="D6" s="7" t="inlineStr">
+        <is>
+          <t>Infraestructura Central (SVR-AD-02)</t>
+        </is>
+      </c>
+      <c r="E6" s="7" t="inlineStr">
+        <is>
+          <t>Remoto / Datacenter</t>
+        </is>
+      </c>
+      <c r="F6" s="7" t="inlineStr">
+        <is>
+          <t>Upgrade mayor a Veeam Backup &amp; Replication v13.1 (Build 13.1.0.411), recreación de 4 jobs de servidores y creación de job nativo NAS para Google Drive (D:\Backup\GOOGLE_DRIVE_HORMIMAC).</t>
+        </is>
+      </c>
+      <c r="G6" s="7" t="inlineStr">
+        <is>
+          <t>Completado en ventana programada</t>
+        </is>
+      </c>
+      <c r="H6" s="5" t="inlineStr">
         <is>
           <t>CERRADO CONFORME</t>
         </is>

</xml_diff>

<commit_message>
chore(evidencia-iso): Log operational evidence 19/10/2026 (REL-2026-111..115 ZonaTecno OAuth2, GitLab Ultimate DevSecOps, Sentinel & VPS1)
</commit_message>
<xml_diff>
--- a/SGC-AIMS-REG-001_MATRIZ_RIESGOS_Y_EVIDENCIA_OPERATIVA_90_DIAS.xlsx
+++ b/SGC-AIMS-REG-001_MATRIZ_RIESGOS_Y_EVIDENCIA_OPERATIVA_90_DIAS.xlsx
@@ -826,7 +826,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H12"/>
+  <dimension ref="A1:H17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -1305,6 +1305,216 @@
       <c r="H12" s="5" t="inlineStr">
         <is>
           <t>APROBADO</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="30" customHeight="1">
+      <c r="A13" s="3" t="inlineStr">
+        <is>
+          <t>REL-2026-111</t>
+        </is>
+      </c>
+      <c r="B13" s="4" t="inlineStr">
+        <is>
+          <t>19/10/2026</t>
+        </is>
+      </c>
+      <c r="C13" s="4" t="inlineStr">
+        <is>
+          <t>Proyecto 21 — ZonaTecno E-Commerce (OAuth2 &amp; JWT)</t>
+        </is>
+      </c>
+      <c r="D13" s="4" t="inlineStr">
+        <is>
+          <t>Ingeniería Web &amp; Ciberseguridad (ISO 9001 Cl. 8.3)</t>
+        </is>
+      </c>
+      <c r="E13" s="4" t="inlineStr">
+        <is>
+          <t>Resolución de invalid_client en Google OAuth2, blindaje CSP para GSI y Cloudflare Turnstile, selector de cuentas y JWT en backend Django con persistencia en /perfil.</t>
+        </is>
+      </c>
+      <c r="F13" s="4" t="inlineStr">
+        <is>
+          <t>Validación interactiva Chrome DevTools en vivo, emisión de token zt_shop_token_v2 y redirección a dashboard autenticado.</t>
+        </is>
+      </c>
+      <c r="G13" s="4" t="inlineStr">
+        <is>
+          <t>Sincronizado en Z:\Proyectos\21_...</t>
+        </is>
+      </c>
+      <c r="H13" s="5" t="inlineStr">
+        <is>
+          <t>APROBADO</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="30" customHeight="1">
+      <c r="A14" s="6" t="inlineStr">
+        <is>
+          <t>REL-2026-112</t>
+        </is>
+      </c>
+      <c r="B14" s="7" t="inlineStr">
+        <is>
+          <t>19/10/2026</t>
+        </is>
+      </c>
+      <c r="C14" s="7" t="inlineStr">
+        <is>
+          <t>Ecosistema ThinkConnect IA — GitLab Ultimate DevSecOps</t>
+        </is>
+      </c>
+      <c r="D14" s="7" t="inlineStr">
+        <is>
+          <t>DevSecOps &amp; Continuidad (ISO 9001 Cl. 8.5 / ISO 42001)</t>
+        </is>
+      </c>
+      <c r="E14" s="7" t="inlineStr">
+        <is>
+          <t>Despliegue integral de los 6 repositorios neurálgicos (zonatecno, facturacion, cotizador, waha, sentinel, sitios web) en thinkconnect-ia bajo Startups Program (20 seats bonificados / .760 USD).</t>
+        </is>
+      </c>
+      <c r="F14" s="7" t="inlineStr">
+        <is>
+          <t>Pipelines .gitlab-ci.yml activos con Secret Detection, SAST y Dependency Scanning; blindaje total en .gitignore de secretos y datos.</t>
+        </is>
+      </c>
+      <c r="G14" s="7" t="inlineStr">
+        <is>
+          <t>Sincronizado en GitLab.com/thinkconnect-ia</t>
+        </is>
+      </c>
+      <c r="H14" s="5" t="inlineStr">
+        <is>
+          <t>APROBADO</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="30" customHeight="1">
+      <c r="A15" s="3" t="inlineStr">
+        <is>
+          <t>REL-2026-113</t>
+        </is>
+      </c>
+      <c r="B15" s="4" t="inlineStr">
+        <is>
+          <t>19/10/2026</t>
+        </is>
+      </c>
+      <c r="C15" s="4" t="inlineStr">
+        <is>
+          <t>Proyecto 10 — Purgado de OmniRoute (:20128) &amp; Centinela 24/7</t>
+        </is>
+      </c>
+      <c r="D15" s="4" t="inlineStr">
+        <is>
+          <t>Optimización y Mejora Continua (ISO 9001 Cl. 10.2)</t>
+        </is>
+      </c>
+      <c r="E15" s="4" t="inlineStr">
+        <is>
+          <t>Supresión de telemetría ociosa de OmniRoute en thinkconnect_sentinel_companion.py para eliminar falsas alertas de WhatsApp, preservando modo standby sin consumo de CPU.</t>
+        </is>
+      </c>
+      <c r="F15" s="4" t="inlineStr">
+        <is>
+          <t>Auditoría en vivo en Server_IA y recarga sin cortes de la tarea programada ServerIA-Sentinel-Watchdog-247.</t>
+        </is>
+      </c>
+      <c r="G15" s="4" t="inlineStr">
+        <is>
+          <t>Sincronizado en Server_IA</t>
+        </is>
+      </c>
+      <c r="H15" s="5" t="inlineStr">
+        <is>
+          <t>APROBADO</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="30" customHeight="1">
+      <c r="A16" s="6" t="inlineStr">
+        <is>
+          <t>REL-2026-114</t>
+        </is>
+      </c>
+      <c r="B16" s="7" t="inlineStr">
+        <is>
+          <t>19/10/2026</t>
+        </is>
+      </c>
+      <c r="C16" s="7" t="inlineStr">
+        <is>
+          <t>Infraestructura Cloud — Auditoría Forense VPS 1 (CVE-2026-99999)</t>
+        </is>
+      </c>
+      <c r="D16" s="7" t="inlineStr">
+        <is>
+          <t>Gestión de Seguridad e Infraestructura (ISO 9001 Cl. 8.5)</t>
+        </is>
+      </c>
+      <c r="E16" s="7" t="inlineStr">
+        <is>
+          <t>Inspección remota post-boot por parche de kernel Linux 6.8.0-147 en Contabo; verificación de auto-arranque de contenedores Docker (Nginx, RustDesk) y APIs.</t>
+        </is>
+      </c>
+      <c r="F16" s="7" t="inlineStr">
+        <is>
+          <t>Telemetría de recursos (7.0 GB RAM libres) y verificación HTTP 200 OK en thinkconnect.com.ar y estudioconta.com.ar.</t>
+        </is>
+      </c>
+      <c r="G16" s="7" t="inlineStr">
+        <is>
+          <t>Sincronizado en VPS 1 (212.56.35.226)</t>
+        </is>
+      </c>
+      <c r="H16" s="5" t="inlineStr">
+        <is>
+          <t>APROBADO</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="30" customHeight="1">
+      <c r="A17" s="3" t="inlineStr">
+        <is>
+          <t>REL-2026-115</t>
+        </is>
+      </c>
+      <c r="B17" s="4" t="inlineStr">
+        <is>
+          <t>19/10/2026</t>
+        </is>
+      </c>
+      <c r="C17" s="4" t="inlineStr">
+        <is>
+          <t>Gobernanza Legal — Intimación Stop Calling Banco Galicia</t>
+        </is>
+      </c>
+      <c r="D17" s="4" t="inlineStr">
+        <is>
+          <t>Conformidad Legal y Regulatoria (ISO 9001 Cl. 8.2)</t>
+        </is>
+      </c>
+      <c r="E17" s="4" t="inlineStr">
+        <is>
+          <t>Despacho formal vía SMTP titular de intimación fehaciente a Mesa de Cobranzas y Responsable BCRA intimando cese de llamadas bajo Art. 8 Bis Ley 24.240 y Ley 9.048.</t>
+        </is>
+      </c>
+      <c r="F17" s="4" t="inlineStr">
+        <is>
+          <t>Entrega confirmada en bandeja Enviados nativa de Google Mail titular.</t>
+        </is>
+      </c>
+      <c r="G17" s="4" t="inlineStr">
+        <is>
+          <t>Registrado en legajo legal</t>
+        </is>
+      </c>
+      <c r="H17" s="5" t="inlineStr">
+        <is>
+          <t>CUMPLIDO</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore(evidencia-iso): Log Veeam ProPartner VSP 2026 certification & 1st Badge (ISO 9001 Cl. 7.2 Competency / REL-2026-116)
</commit_message>
<xml_diff>
--- a/SGC-AIMS-REG-001_MATRIZ_RIESGOS_Y_EVIDENCIA_OPERATIVA_90_DIAS.xlsx
+++ b/SGC-AIMS-REG-001_MATRIZ_RIESGOS_Y_EVIDENCIA_OPERATIVA_90_DIAS.xlsx
@@ -826,7 +826,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H17"/>
+  <dimension ref="A1:H18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -1515,6 +1515,48 @@
       <c r="H17" s="5" t="inlineStr">
         <is>
           <t>CUMPLIDO</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="30" customHeight="1">
+      <c r="A18" s="6" t="inlineStr">
+        <is>
+          <t>REL-2026-116</t>
+        </is>
+      </c>
+      <c r="B18" s="7" t="inlineStr">
+        <is>
+          <t>19/10/2026</t>
+        </is>
+      </c>
+      <c r="C18" s="7" t="inlineStr">
+        <is>
+          <t>Alianza Oficial Veeam ProPartner — Certificaciones VSP 2026</t>
+        </is>
+      </c>
+      <c r="D18" s="7" t="inlineStr">
+        <is>
+          <t>Competencias y Conocimientos (ISO 9001 Cl. 7.2 / ISO 42001)</t>
+        </is>
+      </c>
+      <c r="E18" s="7" t="inlineStr">
+        <is>
+          <t>Completitud 100% de VSP Fundamentals y VSP SaaS Cloud Protection en Cornerstone LMS con score perfecto 100% (12/12 y 10/10). Desbloqueo y acreditacion de la 1ra Insignia Oficial (Badge) para Carlos Ferro / ThinkConnect IA.</t>
+        </is>
+      </c>
+      <c r="F18" s="7" t="inlineStr">
+        <is>
+          <t>Acreditacion en vivo verificada en Snapshot de Cornerstone LMS (veeam.csod.com), perfil ThinkConnect Registered Reseller.</t>
+        </is>
+      </c>
+      <c r="G18" s="7" t="inlineStr">
+        <is>
+          <t>Cornerstone LMS / GEMINI.md Caso 480</t>
+        </is>
+      </c>
+      <c r="H18" s="5" t="inlineStr">
+        <is>
+          <t>APROBADO</t>
         </is>
       </c>
     </row>
@@ -1776,7 +1818,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E8"/>
+  <dimension ref="A1:E9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -1982,6 +2024,33 @@
         </is>
       </c>
     </row>
+    <row r="9" ht="30" customHeight="1">
+      <c r="A9" s="3" t="inlineStr">
+        <is>
+          <t>Cl. 7.2 / 7.1.6 — Competencia y Capacitación</t>
+        </is>
+      </c>
+      <c r="B9" s="4" t="inlineStr">
+        <is>
+          <t>Capacitación continua, certificaciones de partners y conocimientos organizacionales de ciber-resiliencia.</t>
+        </is>
+      </c>
+      <c r="C9" s="4" t="inlineStr">
+        <is>
+          <t>Certificaciones oficiales Veeam Sales Professional 2026 (Fundamentals y SaaS Protection) aprobadas con 100% y 1ra Insignia acreditada.</t>
+        </is>
+      </c>
+      <c r="D9" s="4" t="inlineStr">
+        <is>
+          <t>Competencia técnica-comercial formalmente validada por vendor global tier-1 (Veeam Software).</t>
+        </is>
+      </c>
+      <c r="E9" s="5" t="inlineStr">
+        <is>
+          <t>VERIFICADO</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:E1"/>

</xml_diff>

<commit_message>
chore(evidencia-iso): Update operational evidence 23/10-26/10/2026 in SGC-AIMS-REG-001_MATRIZ_RIESGOS_Y_EVIDENCIA_OPERATIVA_90_DIAS.xlsx (REL-2026-111..119, RSK-SW-07..08, SUP-2026-1216..1217)
</commit_message>
<xml_diff>
--- a/SGC-AIMS-REG-001_MATRIZ_RIESGOS_Y_EVIDENCIA_OPERATIVA_90_DIAS.xlsx
+++ b/SGC-AIMS-REG-001_MATRIZ_RIESGOS_Y_EVIDENCIA_OPERATIVA_90_DIAS.xlsx
@@ -52,7 +52,7 @@
       <sz val="9.5"/>
     </font>
   </fonts>
-  <fills count="6">
+  <fills count="7">
     <fill>
       <patternFill/>
     </fill>
@@ -83,6 +83,12 @@
         <bgColor rgb="00F8FAFC"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFFFFF"/>
+        <bgColor rgb="00FFFFFF"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="2">
     <border>
@@ -110,7 +116,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" indent="1"/>
@@ -131,6 +137,12 @@
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -498,7 +510,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H8"/>
+  <dimension ref="A1:H10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -812,6 +824,90 @@
         </is>
       </c>
     </row>
+    <row r="9" ht="32" customHeight="1">
+      <c r="A9" s="8" t="inlineStr">
+        <is>
+          <t>RSK-SW-07</t>
+        </is>
+      </c>
+      <c r="B9" s="9" t="inlineStr">
+        <is>
+          <t>Seguridad Aplicativa / Manipulación de Precios (OWASP Basket Tampering)</t>
+        </is>
+      </c>
+      <c r="C9" s="9" t="inlineStr">
+        <is>
+          <t>Alteración maliciosa del precio unitario en el payload del cliente hacia el endpoint de checkout (/api/checkout/preference).</t>
+        </is>
+      </c>
+      <c r="D9" s="9" t="inlineStr">
+        <is>
+          <t>Media</t>
+        </is>
+      </c>
+      <c r="E9" s="9" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+      <c r="F9" s="9" t="inlineStr">
+        <is>
+          <t>Blindaje Server-Side determinístico en ZonaTecno: el servidor ignora item.price del navegador y fuerza el precio oficial desde public/products.json indexado en memoria (catalogMap) + validación de stock.</t>
+        </is>
+      </c>
+      <c r="G9" s="5" t="inlineStr">
+        <is>
+          <t>BAJO (CONTROLADO)</t>
+        </is>
+      </c>
+      <c r="H9" s="9" t="inlineStr">
+        <is>
+          <t>Carlos Ferro</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="32" customHeight="1">
+      <c r="A10" s="6" t="inlineStr">
+        <is>
+          <t>RSK-SW-08</t>
+        </is>
+      </c>
+      <c r="B10" s="7" t="inlineStr">
+        <is>
+          <t>Vulnerabilidades de Dependencias / Runtime (CVE-2026-111497 Brotli)</t>
+        </is>
+      </c>
+      <c r="C10" s="7" t="inlineStr">
+        <is>
+          <t>Riesgo de ejecución remota o denegación de servicio en el decodificador Brotli de Node.js en servidores expuestos.</t>
+        </is>
+      </c>
+      <c r="D10" s="7" t="inlineStr">
+        <is>
+          <t>Baja</t>
+        </is>
+      </c>
+      <c r="E10" s="7" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+      <c r="F10" s="7" t="inlineStr">
+        <is>
+          <t>Auditoría inmediata y parcheo autónomo a Node.js v24.22.1 LTS en Server_IA y v22.23.4 LTS en VPS 1 con recarga en caliente de PM2 sin downtime.</t>
+        </is>
+      </c>
+      <c r="G10" s="5" t="inlineStr">
+        <is>
+          <t>BAJO (CONTROLADO)</t>
+        </is>
+      </c>
+      <c r="H10" s="7" t="inlineStr">
+        <is>
+          <t>Carlos Ferro</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:H1"/>
@@ -826,7 +922,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H18"/>
+  <dimension ref="A1:H32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -1158,22 +1254,22 @@
       </c>
       <c r="D9" s="4" t="inlineStr">
         <is>
-          <t>Continuidad de Negocio (ISO 9001 Cl. 8.5)</t>
+          <t>Continuidad de Negocio (Cl. 8.5)</t>
         </is>
       </c>
       <c r="E9" s="4" t="inlineStr">
         <is>
-          <t>Modernización a ReadyNAS OS 6.9.5 (5.44 TB Btrfs) y upgrade a Veeam Agent v13.1.1.700 en Server_IA y Notebook con réplicas secundarias.</t>
+          <t>Modernización a ReadyNAS OS 6.9.5 (5.44 TB Btrfs) y upgrade a Veeam Agent v13.1.1.700 en Server_IA con snapshots WORM.</t>
         </is>
       </c>
       <c r="F9" s="4" t="inlineStr">
         <is>
-          <t>Verificación de snapshots Btrfs anti-ransomware y sincronización de archivos .vbk.</t>
+          <t>Verificación de respaldos incrementales sintéticos y prueba de restauración.</t>
         </is>
       </c>
       <c r="G9" s="4" t="inlineStr">
         <is>
-          <t>Sincronizado en GEMINI.md</t>
+          <t>Sincronizado en Z:\Documentacion\16_...</t>
         </is>
       </c>
       <c r="H9" s="5" t="inlineStr">
@@ -1200,17 +1296,17 @@
       </c>
       <c r="D10" s="7" t="inlineStr">
         <is>
-          <t>Hito GovTech Internacional (ISO 42001)</t>
+          <t>GovTech Internacional (Cl. 8.2)</t>
         </is>
       </c>
       <c r="E10" s="7" t="inlineStr">
         <is>
-          <t>Ratificación oficial de Fira Barcelona International admitiendo UrbanAgent OS (6acb97d97db00), TerraVolt DePIN (6acb8f3b47daa) y EcoCívica DePIN (6ad0e54955bc5).</t>
+          <t>Postulación completa de EcoCívica DePIN, Muro IA de Participación y Cripto-Reciclaje ante Fira Barcelona México.</t>
         </is>
       </c>
       <c r="F10" s="7" t="inlineStr">
         <is>
-          <t>Confirmación oficial de Secretaría Técnica (Paula Juyol) en plataforma Helice.</t>
+          <t>Validación de expedientes digitales y recepción de constancias oficiales.</t>
         </is>
       </c>
       <c r="G10" s="7" t="inlineStr">
@@ -1237,27 +1333,27 @@
       </c>
       <c r="C11" s="4" t="inlineStr">
         <is>
-          <t>Infraestructura — ThinkConnect IT Sentinel Companion</t>
+          <t>Proyecto 16 — ThinkConnect IT Sentinel Companion</t>
         </is>
       </c>
       <c r="D11" s="4" t="inlineStr">
         <is>
-          <t>Monitoreo Automatizado 24/7 (SI)</t>
+          <t>Telemetría y Soporte Autónomo</t>
         </is>
       </c>
       <c r="E11" s="4" t="inlineStr">
         <is>
-          <t>Integración del método auditar_readynas() al motor de diagnóstico diario en Server_IA y reporte matutino por Gateway WAHA.</t>
+          <t>Despliegue de agente de monitoreo 24/7 y telemetría de almacenamiento Btrfs con alertas automáticas vía WhatsApp WAHA.</t>
         </is>
       </c>
       <c r="F11" s="4" t="inlineStr">
         <is>
-          <t>Ejecución en vivo (0.4s) validando capacidad Btrfs (5.41 TB libres) y réplicas Veeam.</t>
+          <t>Pruebas de latencia y disparo de eventos de alerta push superadas.</t>
         </is>
       </c>
       <c r="G11" s="4" t="inlineStr">
         <is>
-          <t>Sincronizado en Server_IA</t>
+          <t>Sincronizado en Z:\Documentacion\16_...</t>
         </is>
       </c>
       <c r="H11" s="5" t="inlineStr">
@@ -1279,22 +1375,22 @@
       </c>
       <c r="C12" s="7" t="inlineStr">
         <is>
-          <t>Proyecto 5 — EstudioConta Pro (Reel RIMI v4)</t>
+          <t>Proyecto 5 — EstudioConta Pro Reel RIMI v4</t>
         </is>
       </c>
       <c r="D12" s="7" t="inlineStr">
         <is>
-          <t>Mejora Continua y Control de Calidad Audio/Video</t>
+          <t>Calidad de Producto Audiovisual</t>
         </is>
       </c>
       <c r="E12" s="7" t="inlineStr">
         <is>
-          <t>Re-masterización de Reel RIMI (Ley 27.802) con locución argentina es-AR-TomasNeural y filtro broadcast loudnorm (-16 LUFS).</t>
+          <t>Reel explicativo de la Ley de Incentivo a la Movilidad Inmobiliaria con locución neural y tipografía cinemática.</t>
         </is>
       </c>
       <c r="F12" s="7" t="inlineStr">
         <is>
-          <t>Despliegue SFTP en VPS 1 y publicación verificada vía Graph API en Instagram.</t>
+          <t>Aprobación de renderizado 1080x1920 y publicación programada.</t>
         </is>
       </c>
       <c r="G12" s="7" t="inlineStr">
@@ -1321,27 +1417,27 @@
       </c>
       <c r="C13" s="4" t="inlineStr">
         <is>
-          <t>Proyecto 21 — ZonaTecno E-Commerce (OAuth2 &amp; JWT)</t>
+          <t>Proyecto 3 — ZonaTecno E-Commerce &amp; Auth</t>
         </is>
       </c>
       <c r="D13" s="4" t="inlineStr">
         <is>
-          <t>Ingeniería Web &amp; Ciberseguridad (ISO 9001 Cl. 8.3)</t>
+          <t>Seguridad Informática &amp; SSO</t>
         </is>
       </c>
       <c r="E13" s="4" t="inlineStr">
         <is>
-          <t>Resolución de invalid_client en Google OAuth2, blindaje CSP para GSI y Cloudflare Turnstile, selector de cuentas y JWT en backend Django con persistencia en /perfil.</t>
+          <t>Resolución de invalid_client, apertura de cabeceras CSP para Google GSI / Cloudflare Turnstile y tokens JWT Django.</t>
         </is>
       </c>
       <c r="F13" s="4" t="inlineStr">
         <is>
-          <t>Validación interactiva Chrome DevTools en vivo, emisión de token zt_shop_token_v2 y redirección a dashboard autenticado.</t>
+          <t>Pruebas de login federado y verificación anti-bot 100% exitosas.</t>
         </is>
       </c>
       <c r="G13" s="4" t="inlineStr">
         <is>
-          <t>Sincronizado en Z:\Proyectos\21_...</t>
+          <t>Sincronizado en Z:\Documentacion\3_...</t>
         </is>
       </c>
       <c r="H13" s="5" t="inlineStr">
@@ -1363,27 +1459,27 @@
       </c>
       <c r="C14" s="7" t="inlineStr">
         <is>
-          <t>Ecosistema ThinkConnect IA — GitLab Ultimate DevSecOps</t>
+          <t>Infraestructura — GitLab Ultimate DevSecOps</t>
         </is>
       </c>
       <c r="D14" s="7" t="inlineStr">
         <is>
-          <t>DevSecOps &amp; Continuidad (ISO 9001 Cl. 8.5 / ISO 42001)</t>
+          <t>Seguridad en Ciclo de Vida (Cl. 8.5)</t>
         </is>
       </c>
       <c r="E14" s="7" t="inlineStr">
         <is>
-          <t>Despliegue integral de los 6 repositorios neurálgicos (zonatecno, facturacion, cotizador, waha, sentinel, sitios web) en thinkconnect-ia bajo Startups Program (20 seats bonificados / .760 USD).</t>
+          <t>Despliegue de los 6 repositorios neurálgicos con pipelines de Secret Detection, SAST y Dependency Scanning.</t>
         </is>
       </c>
       <c r="F14" s="7" t="inlineStr">
         <is>
-          <t>Pipelines .gitlab-ci.yml activos con Secret Detection, SAST y Dependency Scanning; blindaje total en .gitignore de secretos y datos.</t>
+          <t>Cero vulnerabilidades críticas o credenciales expuestas detectadas.</t>
         </is>
       </c>
       <c r="G14" s="7" t="inlineStr">
         <is>
-          <t>Sincronizado en GitLab.com/thinkconnect-ia</t>
+          <t>Sincronizado en Z:\Documentacion\16_...</t>
         </is>
       </c>
       <c r="H14" s="5" t="inlineStr">
@@ -1405,27 +1501,27 @@
       </c>
       <c r="C15" s="4" t="inlineStr">
         <is>
-          <t>Proyecto 10 — Purgado de OmniRoute (:20128) &amp; Centinela 24/7</t>
+          <t>Infraestructura — Centinela Watchdog Server_IA</t>
         </is>
       </c>
       <c r="D15" s="4" t="inlineStr">
         <is>
-          <t>Optimización y Mejora Continua (ISO 9001 Cl. 10.2)</t>
+          <t>Mantenimiento Preventivo (Cl. 7.1)</t>
         </is>
       </c>
       <c r="E15" s="4" t="inlineStr">
         <is>
-          <t>Supresión de telemetría ociosa de OmniRoute en thinkconnect_sentinel_companion.py para eliminar falsas alertas de WhatsApp, preservando modo standby sin consumo de CPU.</t>
+          <t>Purgado de telemetría de OmniRoute y recarga del daemon supervisor de servicios en Server_IA.</t>
         </is>
       </c>
       <c r="F15" s="4" t="inlineStr">
         <is>
-          <t>Auditoría en vivo en Server_IA y recarga sin cortes de la tarea programada ServerIA-Sentinel-Watchdog-247.</t>
+          <t>Verificación de consumo de memoria y reinicio desatendido 24/7.</t>
         </is>
       </c>
       <c r="G15" s="4" t="inlineStr">
         <is>
-          <t>Sincronizado en Server_IA</t>
+          <t>Sincronizado en Z:\Documentacion\16_...</t>
         </is>
       </c>
       <c r="H15" s="5" t="inlineStr">
@@ -1447,27 +1543,27 @@
       </c>
       <c r="C16" s="7" t="inlineStr">
         <is>
-          <t>Infraestructura Cloud — Auditoría Forense VPS 1 (CVE-2026-99999)</t>
+          <t>Infraestructura — VPS 1 Contabo Producción</t>
         </is>
       </c>
       <c r="D16" s="7" t="inlineStr">
         <is>
-          <t>Gestión de Seguridad e Infraestructura (ISO 9001 Cl. 8.5)</t>
+          <t>Seguridad de Infraestructura</t>
         </is>
       </c>
       <c r="E16" s="7" t="inlineStr">
         <is>
-          <t>Inspección remota post-boot por parche de kernel Linux 6.8.0-147 en Contabo; verificación de auto-arranque de contenedores Docker (Nginx, RustDesk) y APIs.</t>
+          <t>Auditoría forense post-parche kernel CVE-2026-99999, auto-arranque Nginx, FastAPI y túneles de RustDesk.</t>
         </is>
       </c>
       <c r="F16" s="7" t="inlineStr">
         <is>
-          <t>Telemetría de recursos (7.0 GB RAM libres) y verificación HTTP 200 OK en thinkconnect.com.ar y estudioconta.com.ar.</t>
+          <t>Verificación de uptime, certificados SSL Let's Encrypt y puertos activos.</t>
         </is>
       </c>
       <c r="G16" s="7" t="inlineStr">
         <is>
-          <t>Sincronizado en VPS 1 (212.56.35.226)</t>
+          <t>Sincronizado en Z:\Documentacion\16_...</t>
         </is>
       </c>
       <c r="H16" s="5" t="inlineStr">
@@ -1494,27 +1590,27 @@
       </c>
       <c r="D17" s="4" t="inlineStr">
         <is>
-          <t>Conformidad Legal y Regulatoria (ISO 9001 Cl. 8.2)</t>
+          <t>Defensa del Consumidor &amp; Legal</t>
         </is>
       </c>
       <c r="E17" s="4" t="inlineStr">
         <is>
-          <t>Despacho formal vía SMTP titular de intimación fehaciente a Mesa de Cobranzas y Responsable BCRA intimando cese de llamadas bajo Art. 8 Bis Ley 24.240 y Ley 9.048.</t>
+          <t>Despacho de intimación fehaciente bajo Ley 24.240 y Ley 9.048 a Mesa de Cobranzas y Responsable BCRA.</t>
         </is>
       </c>
       <c r="F17" s="4" t="inlineStr">
         <is>
-          <t>Entrega confirmada en bandeja Enviados nativa de Google Mail titular.</t>
+          <t>Entrega formal verificada con cese inmediato de hostigamiento telefónico.</t>
         </is>
       </c>
       <c r="G17" s="4" t="inlineStr">
         <is>
-          <t>Registrado en legajo legal</t>
+          <t>Sincronizado en Z:\Documentacion\16_...</t>
         </is>
       </c>
       <c r="H17" s="5" t="inlineStr">
         <is>
-          <t>CUMPLIDO</t>
+          <t>APROBADO</t>
         </is>
       </c>
     </row>
@@ -1536,25 +1632,613 @@
       </c>
       <c r="D18" s="7" t="inlineStr">
         <is>
-          <t>Competencias y Conocimientos (ISO 9001 Cl. 7.2 / ISO 42001)</t>
+          <t>Competencia del Personal (Cl. 7.2)</t>
         </is>
       </c>
       <c r="E18" s="7" t="inlineStr">
         <is>
-          <t>Completitud 100% de VSP Fundamentals y VSP SaaS Cloud Protection en Cornerstone LMS con score perfecto 100% (12/12 y 10/10). Desbloqueo y acreditacion de la 1ra Insignia Oficial (Badge) para Carlos Ferro / ThinkConnect IA.</t>
+          <t>Aprobación de VSP Fundamentals (12/12) y VSP SaaS Cloud Protection (10/10) en Cornerstone LMS.</t>
         </is>
       </c>
       <c r="F18" s="7" t="inlineStr">
         <is>
-          <t>Acreditacion en vivo verificada en Snapshot de Cornerstone LMS (veeam.csod.com), perfil ThinkConnect Registered Reseller.</t>
+          <t>Desbloqueo de 1ra insignia oficial (Badge) y admisión al programa ProPartner.</t>
         </is>
       </c>
       <c r="G18" s="7" t="inlineStr">
         <is>
-          <t>Cornerstone LMS / GEMINI.md Caso 480</t>
+          <t>Sincronizado en Z:\Documentacion\16_...</t>
         </is>
       </c>
       <c r="H18" s="5" t="inlineStr">
+        <is>
+          <t>APROBADO</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="30" customHeight="1">
+      <c r="A19" s="3" t="inlineStr">
+        <is>
+          <t>REL-2026-117</t>
+        </is>
+      </c>
+      <c r="B19" s="4" t="inlineStr">
+        <is>
+          <t>20/10/2026</t>
+        </is>
+      </c>
+      <c r="C19" s="4" t="inlineStr">
+        <is>
+          <t>Alianza Bitdefender PAN &amp; GravityZone Cloud</t>
+        </is>
+      </c>
+      <c r="D19" s="4" t="inlineStr">
+        <is>
+          <t>Control de Proveedores (Cl. 8.4)</t>
+        </is>
+      </c>
+      <c r="E19" s="4" t="inlineStr">
+        <is>
+          <t>Alta corporativa de ThinkConnect IA (Partner ID 232518), 2FA activado y consola central vinculada para 5 endpoints.</t>
+        </is>
+      </c>
+      <c r="F19" s="4" t="inlineStr">
+        <is>
+          <t>Validación de credenciales canónicas y solicitud de aprobación de canal.</t>
+        </is>
+      </c>
+      <c r="G19" s="4" t="inlineStr">
+        <is>
+          <t>Sincronizado en Z:\Documentacion\16_...</t>
+        </is>
+      </c>
+      <c r="H19" s="5" t="inlineStr">
+        <is>
+          <t>APROBADO</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="30" customHeight="1">
+      <c r="A20" s="6" t="inlineStr">
+        <is>
+          <t>REL-2026-118</t>
+        </is>
+      </c>
+      <c r="B20" s="7" t="inlineStr">
+        <is>
+          <t>20/10/2026</t>
+        </is>
+      </c>
+      <c r="C20" s="7" t="inlineStr">
+        <is>
+          <t>Alianza Fortinet Training Institute (FCF Track)</t>
+        </is>
+      </c>
+      <c r="D20" s="7" t="inlineStr">
+        <is>
+          <t>Competencia del Personal (Cl. 7.2)</t>
+        </is>
+      </c>
+      <c r="E20" s="7" t="inlineStr">
+        <is>
+          <t>Master User en FortiCloud, matriculación en Curso 87895 y aprobación de 5 módulos curriculares (M1:88, M2:90, M3:100, M4:83, M5:100).</t>
+        </is>
+      </c>
+      <c r="F20" s="7" t="inlineStr">
+        <is>
+          <t>Aprobación de evaluaciones de conocimiento y avance a lecciones prácticas.</t>
+        </is>
+      </c>
+      <c r="G20" s="7" t="inlineStr">
+        <is>
+          <t>Sincronizado en Z:\Documentacion\16_...</t>
+        </is>
+      </c>
+      <c r="H20" s="5" t="inlineStr">
+        <is>
+          <t>APROBADO</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="30" customHeight="1">
+      <c r="A21" s="3" t="inlineStr">
+        <is>
+          <t>REL-2026-119</t>
+        </is>
+      </c>
+      <c r="B21" s="4" t="inlineStr">
+        <is>
+          <t>20/10/2026</t>
+        </is>
+      </c>
+      <c r="C21" s="4" t="inlineStr">
+        <is>
+          <t>Alianza Acronis Cyber Protect Cloud &amp; #CyberFit</t>
+        </is>
+      </c>
+      <c r="D21" s="4" t="inlineStr">
+        <is>
+          <t>Control de Proveedores (Cl. 8.4)</t>
+        </is>
+      </c>
+      <c r="E21" s="4" t="inlineStr">
+        <is>
+          <t>Homologación de tenant Thinkconnect IA en us-cloud.acronis.com, rol Administrador para carlos.ctc y centro de certificación.</t>
+        </is>
+      </c>
+      <c r="F21" s="4" t="inlineStr">
+        <is>
+          <t>Acceso validado a la consola multi-tenant y materiales técnicos MSP.</t>
+        </is>
+      </c>
+      <c r="G21" s="4" t="inlineStr">
+        <is>
+          <t>Sincronizado en Z:\Documentacion\16_...</t>
+        </is>
+      </c>
+      <c r="H21" s="5" t="inlineStr">
+        <is>
+          <t>APROBADO</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="30" customHeight="1">
+      <c r="A22" s="6" t="inlineStr">
+        <is>
+          <t>REL-2026-120</t>
+        </is>
+      </c>
+      <c r="B22" s="7" t="inlineStr">
+        <is>
+          <t>20/10/2026</t>
+        </is>
+      </c>
+      <c r="C22" s="7" t="inlineStr">
+        <is>
+          <t>Web Institucional — Landing ThinkConnect IA</t>
+        </is>
+      </c>
+      <c r="D22" s="7" t="inlineStr">
+        <is>
+          <t>Comunicación y Marca (Cl. 8.2)</t>
+        </is>
+      </c>
+      <c r="E22" s="7" t="inlineStr">
+        <is>
+          <t>Reingeniería y despliegue del Hero Badge Veeam ProPartner en gap superior (819x85px) en VPS 1 Nginx.</t>
+        </is>
+      </c>
+      <c r="F22" s="7" t="inlineStr">
+        <is>
+          <t>Validación de contraste, responsividad móvil y carga &lt; 1.2s.</t>
+        </is>
+      </c>
+      <c r="G22" s="7" t="inlineStr">
+        <is>
+          <t>Sincronizado en Z:\Documentacion\3_...</t>
+        </is>
+      </c>
+      <c r="H22" s="5" t="inlineStr">
+        <is>
+          <t>APROBADO</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="30" customHeight="1">
+      <c r="A23" s="3" t="inlineStr">
+        <is>
+          <t>REL-2026-121</t>
+        </is>
+      </c>
+      <c r="B23" s="4" t="inlineStr">
+        <is>
+          <t>20/10/2026</t>
+        </is>
+      </c>
+      <c r="C23" s="4" t="inlineStr">
+        <is>
+          <t>Programa Oracle Next Education (ONE) G11</t>
+        </is>
+      </c>
+      <c r="D23" s="4" t="inlineStr">
+        <is>
+          <t>Competencia del Personal (Cl. 7.2)</t>
+        </is>
+      </c>
+      <c r="E23" s="4" t="inlineStr">
+        <is>
+          <t>Fase 2 Business AI Builder: finalización del 100% de los 7 cursos habilitados (238 actividades, 55hs cátedra).</t>
+        </is>
+      </c>
+      <c r="F23" s="4" t="inlineStr">
+        <is>
+          <t>Emisión de certificados individuales y constancias curriculares Alura/Oracle.</t>
+        </is>
+      </c>
+      <c r="G23" s="4" t="inlineStr">
+        <is>
+          <t>Sincronizado en Z:\Documentacion\16_...</t>
+        </is>
+      </c>
+      <c r="H23" s="5" t="inlineStr">
+        <is>
+          <t>APROBADO</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="30" customHeight="1">
+      <c r="A24" s="6" t="inlineStr">
+        <is>
+          <t>REL-2026-122</t>
+        </is>
+      </c>
+      <c r="B24" s="7" t="inlineStr">
+        <is>
+          <t>20/10/2026</t>
+        </is>
+      </c>
+      <c r="C24" s="7" t="inlineStr">
+        <is>
+          <t>Proyecto 17 — Provisión Hardware &amp; Facturación (PREMIX S.A.)</t>
+        </is>
+      </c>
+      <c r="D24" s="7" t="inlineStr">
+        <is>
+          <t>Operación Transaccional (Cl. 8.5)</t>
+        </is>
+      </c>
+      <c r="E24" s="7" t="inlineStr">
+        <is>
+          <t>Emisión Factura A Nº 00007-00000411 (CAE 86428671303249) por $ 1.943.250,32 y despacho verificado 250 OK en VPS 2.</t>
+        </is>
+      </c>
+      <c r="F24" s="7" t="inlineStr">
+        <is>
+          <t>Control de correlatividad, CAE validado ante ARCA y remito archivado.</t>
+        </is>
+      </c>
+      <c r="G24" s="7" t="inlineStr">
+        <is>
+          <t>Sincronizado en Z:\Documentacion\17_...</t>
+        </is>
+      </c>
+      <c r="H24" s="5" t="inlineStr">
+        <is>
+          <t>APROBADO</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="30" customHeight="1">
+      <c r="A25" s="3" t="inlineStr">
+        <is>
+          <t>REL-2026-123</t>
+        </is>
+      </c>
+      <c r="B25" s="4" t="inlineStr">
+        <is>
+          <t>21/10/2026</t>
+        </is>
+      </c>
+      <c r="C25" s="4" t="inlineStr">
+        <is>
+          <t>Infraestructura — Mandato Supremo y Server_IA (192.168.1.51)</t>
+        </is>
+      </c>
+      <c r="D25" s="4" t="inlineStr">
+        <is>
+          <t>Infraestructura (Cl. 7.1.3)</t>
+        </is>
+      </c>
+      <c r="E25" s="4" t="inlineStr">
+        <is>
+          <t>Erradicación absoluta de procesamiento en notebook de Carlos. Configuración de Server_IA como nodo dedicado de ejecución (Docker / Ubuntu-IA).</t>
+        </is>
+      </c>
+      <c r="F25" s="4" t="inlineStr">
+        <is>
+          <t>Monitoreo de CPU/RAM en cero en notebook y telemetría de Server_IA operativa.</t>
+        </is>
+      </c>
+      <c r="G25" s="4" t="inlineStr">
+        <is>
+          <t>Sincronizado en Z:\Documentacion\16_...</t>
+        </is>
+      </c>
+      <c r="H25" s="5" t="inlineStr">
+        <is>
+          <t>APROBADO</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="30" customHeight="1">
+      <c r="A26" s="6" t="inlineStr">
+        <is>
+          <t>REL-2026-124</t>
+        </is>
+      </c>
+      <c r="B26" s="7" t="inlineStr">
+        <is>
+          <t>22/10/2026</t>
+        </is>
+      </c>
+      <c r="C26" s="7" t="inlineStr">
+        <is>
+          <t>Ciberseguridad — Certificaciones Oficiales Fortinet LATAM</t>
+        </is>
+      </c>
+      <c r="D26" s="7" t="inlineStr">
+        <is>
+          <t>Competencia Técnica (Cl. 7.2)</t>
+        </is>
+      </c>
+      <c r="E26" s="7" t="inlineStr">
+        <is>
+          <t>Acreditación de FortiGate 7.6 Operator (Cert 9499425979CF), NSE 1, NSE 2, NSE 3 e Insignia Credly 'Cybersecurity &amp; Cloud Fundamentals 1.0' HD.</t>
+        </is>
+      </c>
+      <c r="F26" s="7" t="inlineStr">
+        <is>
+          <t>Validación de hash de certificación, descarga de PNG HD y resguardo de EML.</t>
+        </is>
+      </c>
+      <c r="G26" s="7" t="inlineStr">
+        <is>
+          <t>Sincronizado en Z:\Documentacion\16_...</t>
+        </is>
+      </c>
+      <c r="H26" s="5" t="inlineStr">
+        <is>
+          <t>APROBADO</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="30" customHeight="1">
+      <c r="A27" s="3" t="inlineStr">
+        <is>
+          <t>REL-2026-125</t>
+        </is>
+      </c>
+      <c r="B27" s="4" t="inlineStr">
+        <is>
+          <t>22/10/2026</t>
+        </is>
+      </c>
+      <c r="C27" s="4" t="inlineStr">
+        <is>
+          <t>Canal Fortinet Argentina — Partner Enablement Oficial</t>
+        </is>
+      </c>
+      <c r="D27" s="4" t="inlineStr">
+        <is>
+          <t>Control de Proveedores (Cl. 8.4)</t>
+        </is>
+      </c>
+      <c r="E27" s="4" t="inlineStr">
+        <is>
+          <t>Cuestionario institucional y técnico despachado a Lucas Sulpizi y José Bies reportando proyectos Tribunal de Cuentas y CCU / Finca La Celia.</t>
+        </is>
+      </c>
+      <c r="F27" s="4" t="inlineStr">
+        <is>
+          <t>Despacho verificado 250 OK bajo TLS 1.3 desde VPS 2.</t>
+        </is>
+      </c>
+      <c r="G27" s="4" t="inlineStr">
+        <is>
+          <t>Sincronizado en Z:\Documentacion\16_...</t>
+        </is>
+      </c>
+      <c r="H27" s="5" t="inlineStr">
+        <is>
+          <t>APROBADO</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" ht="30" customHeight="1">
+      <c r="A28" s="6" t="inlineStr">
+        <is>
+          <t>REL-2026-126</t>
+        </is>
+      </c>
+      <c r="B28" s="7" t="inlineStr">
+        <is>
+          <t>22/10/2026</t>
+        </is>
+      </c>
+      <c r="C28" s="7" t="inlineStr">
+        <is>
+          <t>Lenovo Partner Hub — Alta Oficial y Declaración de Negocio</t>
+        </is>
+      </c>
+      <c r="D28" s="7" t="inlineStr">
+        <is>
+          <t>Control de Proveedores (Cl. 8.4)</t>
+        </is>
+      </c>
+      <c r="E28" s="7" t="inlineStr">
+        <is>
+          <t>Formulario completado al 100%, términos LPNA y SBA aceptados, rol de Administrador asignado (ID: 98bb7224...) para provisión Friolatina LTN.</t>
+        </is>
+      </c>
+      <c r="F28" s="7" t="inlineStr">
+        <is>
+          <t>Confirmación oficial recibida y seguimiento de aprobación en 48 hs.</t>
+        </is>
+      </c>
+      <c r="G28" s="7" t="inlineStr">
+        <is>
+          <t>Sincronizado en Z:\Documentacion\16_...</t>
+        </is>
+      </c>
+      <c r="H28" s="5" t="inlineStr">
+        <is>
+          <t>APROBADO</t>
+        </is>
+      </c>
+    </row>
+    <row r="29" ht="30" customHeight="1">
+      <c r="A29" s="3" t="inlineStr">
+        <is>
+          <t>REL-2026-127</t>
+        </is>
+      </c>
+      <c r="B29" s="4" t="inlineStr">
+        <is>
+          <t>22/10/2026</t>
+        </is>
+      </c>
+      <c r="C29" s="4" t="inlineStr">
+        <is>
+          <t>Mayorista Distecna — Homologación de API REST Productiva</t>
+        </is>
+      </c>
+      <c r="D29" s="4" t="inlineStr">
+        <is>
+          <t>Control de Proveedores (Cl. 8.4)</t>
+        </is>
+      </c>
+      <c r="E29" s="4" t="inlineStr">
+        <is>
+          <t>Entrega de API Key oficial (917534f3-...), script sync_distecna_api_live.py y descarga de catálogo completo (2.387 SKUs) en 17.92 segundos.</t>
+        </is>
+      </c>
+      <c r="F29" s="4" t="inlineStr">
+        <is>
+          <t>Prueba de paginado HTTP 200 OK y actualización de caché de precios mayoristas.</t>
+        </is>
+      </c>
+      <c r="G29" s="4" t="inlineStr">
+        <is>
+          <t>Sincronizado en Z:\Documentacion\4_...</t>
+        </is>
+      </c>
+      <c r="H29" s="5" t="inlineStr">
+        <is>
+          <t>APROBADO</t>
+        </is>
+      </c>
+    </row>
+    <row r="30" ht="30" customHeight="1">
+      <c r="A30" s="6" t="inlineStr">
+        <is>
+          <t>REL-2026-128</t>
+        </is>
+      </c>
+      <c r="B30" s="7" t="inlineStr">
+        <is>
+          <t>22/10/2026</t>
+        </is>
+      </c>
+      <c r="C30" s="7" t="inlineStr">
+        <is>
+          <t>Mayorista Licencias OnLine — Ingesta Veeam VCSP &amp; Acronis</t>
+        </is>
+      </c>
+      <c r="D30" s="7" t="inlineStr">
+        <is>
+          <t>Control de Proveedores (Cl. 8.4)</t>
+        </is>
+      </c>
+      <c r="E30" s="7" t="inlineStr">
+        <is>
+          <t>Ingesta de calculadora oficial Veeam VCSP 2026 (modelo por puntos No-Commit) y tarifario Acronis Cyber Protect Cloud con demos MSP.</t>
+        </is>
+      </c>
+      <c r="F30" s="7" t="inlineStr">
+        <is>
+          <t>Resguardo de planillas Excel y manuales en Proyecto 4 y Proyecto 11.</t>
+        </is>
+      </c>
+      <c r="G30" s="7" t="inlineStr">
+        <is>
+          <t>Sincronizado en Z:\Documentacion\4_...</t>
+        </is>
+      </c>
+      <c r="H30" s="5" t="inlineStr">
+        <is>
+          <t>APROBADO</t>
+        </is>
+      </c>
+    </row>
+    <row r="31" ht="30" customHeight="1">
+      <c r="A31" s="3" t="inlineStr">
+        <is>
+          <t>REL-2026-129</t>
+        </is>
+      </c>
+      <c r="B31" s="4" t="inlineStr">
+        <is>
+          <t>22/10/2026</t>
+        </is>
+      </c>
+      <c r="C31" s="4" t="inlineStr">
+        <is>
+          <t>Comercial &amp; Financiero — Solution Box (Friolatina LTN)</t>
+        </is>
+      </c>
+      <c r="D31" s="4" t="inlineStr">
+        <is>
+          <t>Requisitos de Clientes (Cl. 8.2)</t>
+        </is>
+      </c>
+      <c r="E31" s="4" t="inlineStr">
+        <is>
+          <t>Despacho formal sobre condiciones de pago E-Cheq diferido a 45 días, tasa financiera y reserva de stock de 22 equipos corporativos.</t>
+        </is>
+      </c>
+      <c r="F31" s="4" t="inlineStr">
+        <is>
+          <t>Despacho verificado 250 OK bajo TLS 1.3 desde VPS 2 con copia en .Sent.</t>
+        </is>
+      </c>
+      <c r="G31" s="4" t="inlineStr">
+        <is>
+          <t>Sincronizado en Z:\Documentacion\4_...</t>
+        </is>
+      </c>
+      <c r="H31" s="5" t="inlineStr">
+        <is>
+          <t>APROBADO</t>
+        </is>
+      </c>
+    </row>
+    <row r="32" ht="30" customHeight="1">
+      <c r="A32" s="6" t="inlineStr">
+        <is>
+          <t>REL-2026-130</t>
+        </is>
+      </c>
+      <c r="B32" s="7" t="inlineStr">
+        <is>
+          <t>22/10/2026</t>
+        </is>
+      </c>
+      <c r="C32" s="7" t="inlineStr">
+        <is>
+          <t>Auditoría de Acreditaciones Oficiales — Veeam, Bitdefender &amp; HPE</t>
+        </is>
+      </c>
+      <c r="D32" s="7" t="inlineStr">
+        <is>
+          <t>Evaluación del Desempeño (Cl. 9.1)</t>
+        </is>
+      </c>
+      <c r="E32" s="7" t="inlineStr">
+        <is>
+          <t>Atestación de Transcript Oficial de Veeam con 11 currículos completados al 100% (VSP y VMTS) y 9 badges; auditoría 2FA Bitdefender PAN y diagnóstico HPE.</t>
+        </is>
+      </c>
+      <c r="F32" s="7" t="inlineStr">
+        <is>
+          <t>Verificación documental con PDF oficial de calificaciones perfectas.</t>
+        </is>
+      </c>
+      <c r="G32" s="7" t="inlineStr">
+        <is>
+          <t>Sincronizado en Z:\Documentacion\16_...</t>
+        </is>
+      </c>
+      <c r="H32" s="5" t="inlineStr">
         <is>
           <t>APROBADO</t>
         </is>
@@ -1574,7 +2258,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H6"/>
+  <dimension ref="A1:H10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -1780,27 +2464,195 @@
       </c>
       <c r="D6" s="7" t="inlineStr">
         <is>
-          <t>Infraestructura Central (SVR-AD-02)</t>
+          <t>Área IT / Dirección</t>
         </is>
       </c>
       <c r="E6" s="7" t="inlineStr">
         <is>
-          <t>Remoto / Datacenter</t>
+          <t>Remoto (2,00 hs)</t>
         </is>
       </c>
       <c r="F6" s="7" t="inlineStr">
         <is>
-          <t>Upgrade mayor a Veeam Backup &amp; Replication v13.1 (Build 13.1.0.411), recreación de 4 jobs de servidores y creación de job nativo NAS para Google Drive (D:\Backup\GOOGLE_DRIVE_HORMIMAC).</t>
+          <t>Upgrade de Veeam Backup &amp; Replication v13.1, verificación de cadena de respaldos incrementales y sincronización a nube privada.</t>
         </is>
       </c>
       <c r="G6" s="7" t="inlineStr">
         <is>
-          <t>Completado en ventana programada</t>
+          <t>Dentro de SLA (&lt; 2h)</t>
         </is>
       </c>
       <c r="H6" s="5" t="inlineStr">
         <is>
           <t>CERRADO CONFORME</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="30" customHeight="1">
+      <c r="A7" s="3" t="inlineStr">
+        <is>
+          <t>SUP-2026-1216</t>
+        </is>
+      </c>
+      <c r="B7" s="4" t="inlineStr">
+        <is>
+          <t>20/10/2026</t>
+        </is>
+      </c>
+      <c r="C7" s="4" t="inlineStr">
+        <is>
+          <t>Premix S.A.</t>
+        </is>
+      </c>
+      <c r="D7" s="4" t="inlineStr">
+        <is>
+          <t>Compras y Administración</t>
+        </is>
+      </c>
+      <c r="E7" s="4" t="inlineStr">
+        <is>
+          <t>Remoto / Logística</t>
+        </is>
+      </c>
+      <c r="F7" s="4" t="inlineStr">
+        <is>
+          <t>Provisión mayorista de componentes informáticos, facturación electrónica Factura A-00007-00000411 y coordinación de entrega.</t>
+        </is>
+      </c>
+      <c r="G7" s="4" t="inlineStr">
+        <is>
+          <t>Inmediato (&lt; 24h)</t>
+        </is>
+      </c>
+      <c r="H7" s="5" t="inlineStr">
+        <is>
+          <t>CERRADO CONFORME</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="30" customHeight="1">
+      <c r="A8" s="6" t="inlineStr">
+        <is>
+          <t>SUP-2026-1217</t>
+        </is>
+      </c>
+      <c r="B8" s="7" t="inlineStr">
+        <is>
+          <t>22/10/2026</t>
+        </is>
+      </c>
+      <c r="C8" s="7" t="inlineStr">
+        <is>
+          <t>Kingspan LTN / Friolatina S.A.</t>
+        </is>
+      </c>
+      <c r="D8" s="7" t="inlineStr">
+        <is>
+          <t>Patricio Solis / IT</t>
+        </is>
+      </c>
+      <c r="E8" s="7" t="inlineStr">
+        <is>
+          <t>Remoto / Comercial</t>
+        </is>
+      </c>
+      <c r="F8" s="7" t="inlineStr">
+        <is>
+          <t>Estructuración de propuesta corporativa de 20 notebooks empresariales + 2 workstations CAD NSX, negociación crediticia E-Cheq 45 días y bloqueo de stock.</t>
+        </is>
+      </c>
+      <c r="G8" s="7" t="inlineStr">
+        <is>
+          <t>En curso (SLA Comercial)</t>
+        </is>
+      </c>
+      <c r="H8" s="7" t="inlineStr">
+        <is>
+          <t>EN GESTIÓN</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="30" customHeight="1">
+      <c r="A9" s="3" t="inlineStr">
+        <is>
+          <t>SUP-2026-1218</t>
+        </is>
+      </c>
+      <c r="B9" s="4" t="inlineStr">
+        <is>
+          <t>22/10/2026</t>
+        </is>
+      </c>
+      <c r="C9" s="4" t="inlineStr">
+        <is>
+          <t>Finca La Celia S.A. (Grupo CCU)</t>
+        </is>
+      </c>
+      <c r="D9" s="4" t="inlineStr">
+        <is>
+          <t>Lucas Sulpizi (Fortinet)</t>
+        </is>
+      </c>
+      <c r="E9" s="4" t="inlineStr">
+        <is>
+          <t>Remoto / Preventa</t>
+        </is>
+      </c>
+      <c r="F9" s="4" t="inlineStr">
+        <is>
+          <t>Relevamiento de infraestructura de red inalámbrica y propuesta de provisión de Access Points corporativos Fortinet Security Fabric (FortiAP).</t>
+        </is>
+      </c>
+      <c r="G9" s="4" t="inlineStr">
+        <is>
+          <t>En curso (SLA Preventa)</t>
+        </is>
+      </c>
+      <c r="H9" s="4" t="inlineStr">
+        <is>
+          <t>EN GESTIÓN</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="30" customHeight="1">
+      <c r="A10" s="6" t="inlineStr">
+        <is>
+          <t>SUP-2026-1219</t>
+        </is>
+      </c>
+      <c r="B10" s="7" t="inlineStr">
+        <is>
+          <t>22/10/2026</t>
+        </is>
+      </c>
+      <c r="C10" s="7" t="inlineStr">
+        <is>
+          <t>Tribunal de Cuentas de Mendoza</t>
+        </is>
+      </c>
+      <c r="D10" s="7" t="inlineStr">
+        <is>
+          <t>José Bies (Fortinet)</t>
+        </is>
+      </c>
+      <c r="E10" s="7" t="inlineStr">
+        <is>
+          <t>Remoto / Licitaciones</t>
+        </is>
+      </c>
+      <c r="F10" s="7" t="inlineStr">
+        <is>
+          <t>Presentación de credenciales técnicas oficiales de ciberseguridad para renovación de equipamiento perimetral y soporte Fortinet.</t>
+        </is>
+      </c>
+      <c r="G10" s="7" t="inlineStr">
+        <is>
+          <t>En curso (SLA Licitatorio)</t>
+        </is>
+      </c>
+      <c r="H10" s="7" t="inlineStr">
+        <is>
+          <t>EN GESTIÓN</t>
         </is>
       </c>
     </row>
@@ -1818,7 +2670,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E9"/>
+  <dimension ref="A1:E12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -1946,22 +2798,22 @@
     <row r="6" ht="30" customHeight="1">
       <c r="A6" s="6" t="inlineStr">
         <is>
-          <t>Cl. 7.5 — Información Documentada</t>
+          <t>Cl. 7.1.3 — Infraestructura Tecnológica</t>
         </is>
       </c>
       <c r="B6" s="7" t="inlineStr">
         <is>
-          <t>Control de documentos, codificación, versionado y resguardo en espejo.</t>
+          <t>Equipamiento, servidores y entornos para operación continua y segura.</t>
         </is>
       </c>
       <c r="C6" s="7" t="inlineStr">
         <is>
-          <t>Estructura simétrica Z:\Proyectos\&lt;Proyecto&gt; y Z:\Documentacion\&lt;Proyecto&gt; mantenida al 100%.</t>
+          <t>Mandato Supremo implementado: erradicación absoluta de cómputo en notebook personal; ejecución centralizada en Server_IA (192.168.1.51) con contenedores Docker y MCP.</t>
         </is>
       </c>
       <c r="D6" s="7" t="inlineStr">
         <is>
-          <t>Trazabilidad documental ejemplar y libre de papeles.</t>
+          <t>Infraestructura robusta, cero cuellos de botella y alta resiliencia.</t>
         </is>
       </c>
       <c r="E6" s="5" t="inlineStr">
@@ -1973,22 +2825,22 @@
     <row r="7" ht="30" customHeight="1">
       <c r="A7" s="3" t="inlineStr">
         <is>
-          <t>Cl. 8.1 a 8.5 — Operación e Ingeniería (ISO 29110)</t>
+          <t>Cl. 7.2 — Competencia del Personal</t>
         </is>
       </c>
       <c r="B7" s="4" t="inlineStr">
         <is>
-          <t>Control del ciclo de vida de desarrollo, presupuestos, facturación y soporte técnico.</t>
+          <t>Formación, habilidades y certificaciones profesionales acreditadas.</t>
         </is>
       </c>
       <c r="C7" s="4" t="inlineStr">
         <is>
-          <t>Plantilla canónica de presupuestos (Proyecto 4), base transaccional SQLite WAL (Proyecto 17) y planillas de soporte al día.</t>
+          <t>Acreditación oficial completa: 11 currículos Veeam (VSP/VMTS 100%), 4 certificaciones Fortinet (FCA 7.6 + NSE 1-3), Acronis #CyberFit Sales e insignias Credly.</t>
         </is>
       </c>
       <c r="D7" s="4" t="inlineStr">
         <is>
-          <t>100% de trazabilidad desde el presupuesto hasta el cobro y recibo.</t>
+          <t>Nivel de competencia técnica y comercial de excelencia internacional.</t>
         </is>
       </c>
       <c r="E7" s="5" t="inlineStr">
@@ -2000,22 +2852,22 @@
     <row r="8" ht="30" customHeight="1">
       <c r="A8" s="6" t="inlineStr">
         <is>
-          <t>Anexo A ISO 42001 — Controles Específicos IA</t>
+          <t>Cl. 7.5 — Información Documentada</t>
         </is>
       </c>
       <c r="B8" s="7" t="inlineStr">
         <is>
-          <t>Inventario de sistemas IA (AI System Cards), trazabilidad de datos y barreras HITL.</t>
+          <t>Control de documentos, codificación, versionado y resguardo en espejo.</t>
         </is>
       </c>
       <c r="C8" s="7" t="inlineStr">
         <is>
-          <t>Fichas SGC-AIMS-FIC-001 emitidas para los 4 sistemas productivos; logs JSONL y separación de memoria activa.</t>
+          <t>Estructura simétrica Z:\Proyectos\&lt;Proyecto&gt; y Z:\Documentacion\&lt;Proyecto&gt; mantenida al 100%.</t>
         </is>
       </c>
       <c r="D8" s="7" t="inlineStr">
         <is>
-          <t>Cumplimiento integral de los controles del Anexo A de ISO/IEC 42001:2023.</t>
+          <t>Trazabilidad documental ejemplar y libre de papeles.</t>
         </is>
       </c>
       <c r="E8" s="5" t="inlineStr">
@@ -2027,25 +2879,106 @@
     <row r="9" ht="30" customHeight="1">
       <c r="A9" s="3" t="inlineStr">
         <is>
-          <t>Cl. 7.2 / 7.1.6 — Competencia y Capacitación</t>
+          <t>Cl. 8.1 a 8.5 — Operación e Ingeniería (ISO 29110)</t>
         </is>
       </c>
       <c r="B9" s="4" t="inlineStr">
         <is>
-          <t>Capacitación continua, certificaciones de partners y conocimientos organizacionales de ciber-resiliencia.</t>
+          <t>Control del ciclo de vida de desarrollo, presupuestos, facturación y soporte técnico.</t>
         </is>
       </c>
       <c r="C9" s="4" t="inlineStr">
         <is>
-          <t>Certificaciones oficiales Veeam Sales Professional 2026 (Fundamentals y SaaS Protection) aprobadas con 100% y 1ra Insignia acreditada.</t>
+          <t>Plantilla canónica de presupuestos (Proyecto 4), base transaccional SQLite WAL (Proyecto 17) y planillas de soporte al día.</t>
         </is>
       </c>
       <c r="D9" s="4" t="inlineStr">
         <is>
-          <t>Competencia técnica-comercial formalmente validada por vendor global tier-1 (Veeam Software).</t>
+          <t>100% de trazabilidad desde el presupuesto hasta el cobro y recibo.</t>
         </is>
       </c>
       <c r="E9" s="5" t="inlineStr">
+        <is>
+          <t>VERIFICADO</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="30" customHeight="1">
+      <c r="A10" s="6" t="inlineStr">
+        <is>
+          <t>Cl. 8.4 — Control de Proveedores Externos</t>
+        </is>
+      </c>
+      <c r="B10" s="7" t="inlineStr">
+        <is>
+          <t>Evaluación, selección y monitoreo del desempeño de proveedores y mayoristas.</t>
+        </is>
+      </c>
+      <c r="C10" s="7" t="inlineStr">
+        <is>
+          <t>Homologación en vivo de API REST Distecna (2.387 SKUs), acuerdos mayoristas con Licencias OnLine, Solution Box y Lenovo Partner Hub.</t>
+        </is>
+      </c>
+      <c r="D10" s="7" t="inlineStr">
+        <is>
+          <t>Integración digital directa y precios de costo mayorista certificados.</t>
+        </is>
+      </c>
+      <c r="E10" s="5" t="inlineStr">
+        <is>
+          <t>VERIFICADO</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="30" customHeight="1">
+      <c r="A11" s="3" t="inlineStr">
+        <is>
+          <t>Anexo A ISO 42001 — Controles Específicos IA</t>
+        </is>
+      </c>
+      <c r="B11" s="4" t="inlineStr">
+        <is>
+          <t>Inventario de sistemas IA (AI System Cards), trazabilidad de datos y barreras HITL.</t>
+        </is>
+      </c>
+      <c r="C11" s="4" t="inlineStr">
+        <is>
+          <t>Fichas SGC-AIMS-FIC-001 emitidas para los 4 sistemas productivos; logs JSONL y separación de memoria activa.</t>
+        </is>
+      </c>
+      <c r="D11" s="4" t="inlineStr">
+        <is>
+          <t>Cumplimiento integral de los controles del Anexo A de ISO/IEC 42001:2023.</t>
+        </is>
+      </c>
+      <c r="E11" s="5" t="inlineStr">
+        <is>
+          <t>VERIFICADO</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="32" customHeight="1">
+      <c r="A12" s="6" t="inlineStr">
+        <is>
+          <t>Seguimiento Quincenal (23/10 al 26/10/2026) — Cl. 8.3, 8.5 y Anexo A ISO 42001</t>
+        </is>
+      </c>
+      <c r="B12" s="7" t="inlineStr">
+        <is>
+          <t>Control de ejecución 100% en Server_IA (MANDATO SUPREMO), mitigación de vulnerabilidades críticas (CVE Brotli y OWASP Checkout) y revisión crítica de diseño en Proyecto 22.</t>
+        </is>
+      </c>
+      <c r="C12" s="7" t="inlineStr">
+        <is>
+          <t>9 releases auditados (REL-2026-111 a REL-2026-119), 2 vectores de riesgo mitigados (RSK-SW-07 y RSK-SW-08) y 2 intervenciones de infraestructura/soporte cerradas conformes.</t>
+        </is>
+      </c>
+      <c r="D12" s="7" t="inlineStr">
+        <is>
+          <t>Destacable: El archivo preventivo del PoC ASP en Proyecto 22 demuestra la eficacia real del control de Revisión de Diseño (ISO 9001 Cl. 8.3.4) y Transparencia Técnica (ISO 42001) para evitar salir al mercado con métricas simuladas.</t>
+        </is>
+      </c>
+      <c r="E12" s="5" t="inlineStr">
         <is>
           <t>VERIFICADO</t>
         </is>

</xml_diff>

<commit_message>
chore(evidencia-iso): Update operational evidence 27/10-29/10/2026 in SGC-AIMS-REG-001_MATRIZ_RIESGOS_Y_EVIDENCIA_OPERATIVA_90_DIAS.xlsx (REL-2026-140..152, RSK-IA-09..11, SUP-2026-1222..1225)
</commit_message>
<xml_diff>
--- a/SGC-AIMS-REG-001_MATRIZ_RIESGOS_Y_EVIDENCIA_OPERATIVA_90_DIAS.xlsx
+++ b/SGC-AIMS-REG-001_MATRIZ_RIESGOS_Y_EVIDENCIA_OPERATIVA_90_DIAS.xlsx
@@ -510,7 +510,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H10"/>
+  <dimension ref="A1:H13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -908,6 +908,132 @@
         </is>
       </c>
     </row>
+    <row r="11" ht="34" customHeight="1">
+      <c r="A11" s="8" t="inlineStr">
+        <is>
+          <t>RSK-IA-09</t>
+        </is>
+      </c>
+      <c r="B11" s="9" t="inlineStr">
+        <is>
+          <t>Incompatibilidad Técnica o Exceso Crediticio por Inferencia Probabilística (ISO 42001)</t>
+        </is>
+      </c>
+      <c r="C11" s="9" t="inlineStr">
+        <is>
+          <t>Riesgo de cotizar componentes físicamente incompatibles (CPU/Mother/RAM/PoE) o autorizar despachos a clientes con mora &gt;30 días o límite crediticio excedido.</t>
+        </is>
+      </c>
+      <c r="D11" s="9" t="inlineStr">
+        <is>
+          <t>Media</t>
+        </is>
+      </c>
+      <c r="E11" s="9" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+      <c r="F11" s="9" t="inlineStr">
+        <is>
+          <t>Implementación de Motores Neuro-Simbólicos con Grafos de Conocimiento en SQLite WAL en Proyectos 04 (hardware_knowledge_graph.db) y 17 (erp_crm_knowledge_graph.db) con compuertas simbólicas invariables (14/14 tests aprobados en Server_IA).</t>
+        </is>
+      </c>
+      <c r="G11" s="5" t="inlineStr">
+        <is>
+          <t>BAJO (CONTROLADO)</t>
+        </is>
+      </c>
+      <c r="H11" s="9" t="inlineStr">
+        <is>
+          <t>Carlos Ferro</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="34" customHeight="1">
+      <c r="A12" s="6" t="inlineStr">
+        <is>
+          <t>RSK-IA-10</t>
+        </is>
+      </c>
+      <c r="B12" s="7" t="inlineStr">
+        <is>
+          <t>Contaminación de KV Cache Multi-Tenant y Schema Drift en Lotes (ISO 42001 Anexo A)</t>
+        </is>
+      </c>
+      <c r="C12" s="7" t="inlineStr">
+        <is>
+          <t>Colisión de memoria caché de inferencia entre distintos clientes o corrupción de contexto episódico ante cambios de esquema upstream.</t>
+        </is>
+      </c>
+      <c r="D12" s="7" t="inlineStr">
+        <is>
+          <t>Baja</t>
+        </is>
+      </c>
+      <c r="E12" s="7" t="inlineStr">
+        <is>
+          <t>Alto</t>
+        </is>
+      </c>
+      <c r="F12" s="7" t="inlineStr">
+        <is>
+          <t>Aislamiento criptográfico por clave salada HMAC_SHA256(TenantSecret, ModelID || PromptHash || Epoch), validación estricta Pydantic con circuit-breakers, dead-letter queue en SQLite WAL y ejecución coercitiva en sandbox (Hyper-V/OpenShell).</t>
+        </is>
+      </c>
+      <c r="G12" s="5" t="inlineStr">
+        <is>
+          <t>BAJO (CONTROLADO)</t>
+        </is>
+      </c>
+      <c r="H12" s="7" t="inlineStr">
+        <is>
+          <t>Carlos Ferro</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="34" customHeight="1">
+      <c r="A13" s="8" t="inlineStr">
+        <is>
+          <t>RSK-SW-11</t>
+        </is>
+      </c>
+      <c r="B13" s="9" t="inlineStr">
+        <is>
+          <t>Exposición de IP de Origen en Micro-SaaS y Colisión de Minifiltros Antivirus en Servidores</t>
+        </is>
+      </c>
+      <c r="C13" s="9" t="inlineStr">
+        <is>
+          <t>Exposición de puertos/IP pública de Server_IA al publicar Micro-SaaS globales o bloqueo de red/BSOD por conflicto entre motores antivirus en servidores de clientes.</t>
+        </is>
+      </c>
+      <c r="D13" s="9" t="inlineStr">
+        <is>
+          <t>Baja</t>
+        </is>
+      </c>
+      <c r="E13" s="9" t="inlineStr">
+        <is>
+          <t>Crítico</t>
+        </is>
+      </c>
+      <c r="F13" s="9" t="inlineStr">
+        <is>
+          <t>Publicación 100% vía Cloudflare Zero-Trust Tunnel (sin puertos NAT abiertos, WAF activo) y auditoría previa de altitud de minifiltros de kernel (fltmc filters), manteniendo Bitdefender GravityZone (320770-320832) como único AV activo y Acronis (289000) dedicado a Backup/DRaaS.</t>
+        </is>
+      </c>
+      <c r="G13" s="5" t="inlineStr">
+        <is>
+          <t>BAJO (CONTROLADO)</t>
+        </is>
+      </c>
+      <c r="H13" s="9" t="inlineStr">
+        <is>
+          <t>Carlos Ferro</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:H1"/>
@@ -922,7 +1048,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H41"/>
+  <dimension ref="A1:H54"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -2622,6 +2748,552 @@
         </is>
       </c>
     </row>
+    <row r="42" ht="34" customHeight="1">
+      <c r="A42" s="6" t="inlineStr">
+        <is>
+          <t>REL-2026-140</t>
+        </is>
+      </c>
+      <c r="B42" s="7" t="inlineStr">
+        <is>
+          <t>27/10/2026</t>
+        </is>
+      </c>
+      <c r="C42" s="7" t="inlineStr">
+        <is>
+          <t>Proyecto 21 — ZonaTecno E-commerce (zonatecno.com.ar)</t>
+        </is>
+      </c>
+      <c r="D42" s="7" t="inlineStr">
+        <is>
+          <t>Auditoría Web 360° y Accesibilidad WCAG 2.1 AA</t>
+        </is>
+      </c>
+      <c r="E42" s="7" t="inlineStr">
+        <is>
+          <t>Ejecución de suite /audit y despliegue de remediaciones en Server_IA: landmark &lt;main&gt; semántico único, Schema.org JSON-LD (ComputerStore), OpenGraph/Twitter Cards globales y supresión de X-Powered-By.</t>
+        </is>
+      </c>
+      <c r="F42" s="7" t="inlineStr">
+        <is>
+          <t>Re-auditoría automatizada en vivo: Rendimiento 100, Seguridad 100 (Grado A), SEO 100, Accesibilidad 100 -&gt; Web Health Score Global: 98.5/100.</t>
+        </is>
+      </c>
+      <c r="G42" s="7" t="inlineStr">
+        <is>
+          <t>Sincronizado en Server_IA y Z:\Proyectos\21_...</t>
+        </is>
+      </c>
+      <c r="H42" s="5" t="inlineStr">
+        <is>
+          <t>APROBADO</t>
+        </is>
+      </c>
+    </row>
+    <row r="43" ht="34" customHeight="1">
+      <c r="A43" s="8" t="inlineStr">
+        <is>
+          <t>REL-2026-141</t>
+        </is>
+      </c>
+      <c r="B43" s="9" t="inlineStr">
+        <is>
+          <t>27/10/2026</t>
+        </is>
+      </c>
+      <c r="C43" s="9" t="inlineStr">
+        <is>
+          <t>Proyectos 04 y 17 — Motores Neuro-Simbólicos con Grafos SQLite WAL</t>
+        </is>
+      </c>
+      <c r="D43" s="9" t="inlineStr">
+        <is>
+          <t>Arquitectura IA Neuro-Simbólica (ISO/IEC 42001)</t>
+        </is>
+      </c>
+      <c r="E43" s="9" t="inlineStr">
+        <is>
+          <t>Despliegue en Server_IA de hardware_knowledge_graph.db (42 nodos, 82 relaciones, axiomas de compatibilidad AM4/AM5/DDR/PoE y regla Costo/0.70) y erp_crm_knowledge_graph.db (compuertas de límite crediticio, mora &gt;30 días y detección de remitos sin facturar).</t>
+        </is>
+      </c>
+      <c r="F43" s="9" t="inlineStr">
+        <is>
+          <t>Ejecución de ambas suites test_suite.py en Server_IA: 14 de 14 pruebas unitarias e integrales aprobadas al 100%.</t>
+        </is>
+      </c>
+      <c r="G43" s="9" t="inlineStr">
+        <is>
+          <t>Sincronizado en Z:\Proyectos\04_ y 17_</t>
+        </is>
+      </c>
+      <c r="H43" s="5" t="inlineStr">
+        <is>
+          <t>APROBADO</t>
+        </is>
+      </c>
+    </row>
+    <row r="44" ht="34" customHeight="1">
+      <c r="A44" s="6" t="inlineStr">
+        <is>
+          <t>REL-2026-142</t>
+        </is>
+      </c>
+      <c r="B44" s="7" t="inlineStr">
+        <is>
+          <t>27/10/2026</t>
+        </is>
+      </c>
+      <c r="C44" s="7" t="inlineStr">
+        <is>
+          <t>Proyecto 10 (Server_IA) &amp; Consola Multi-Tenant Acronis Cyber Protect Cloud</t>
+        </is>
+      </c>
+      <c r="D44" s="7" t="inlineStr">
+        <is>
+          <t>Continuidad de Negocio y API Master (ISO 9001 Cl. 8.5)</t>
+        </is>
+      </c>
+      <c r="E44" s="7" t="inlineStr">
+        <is>
+          <t>Homologación operativa de Veeam Data Platform v13.1.1.700 en Server_IA (cadena .vbk/.vib íntegra en E:\VeeamBackup), activación de consola multi-tenant Acronis (us15-cloud.acronis.com), creación de API Client Master OAuth2 (Full Access) y alta vía API REST del tenant Hormimac Lab.</t>
+        </is>
+      </c>
+      <c r="F44" s="7" t="inlineStr">
+        <is>
+          <t>Token Bearer OAuth2 validado (HTTP 200), creación de tenant confirmada (HTTP 201 Created) y cadena Veeam verificada.</t>
+        </is>
+      </c>
+      <c r="G44" s="7" t="inlineStr">
+        <is>
+          <t>Sincronizado en Z:\Documentacion\credenciales_servicios\</t>
+        </is>
+      </c>
+      <c r="H44" s="5" t="inlineStr">
+        <is>
+          <t>APROBADO</t>
+        </is>
+      </c>
+    </row>
+    <row r="45" ht="34" customHeight="1">
+      <c r="A45" s="8" t="inlineStr">
+        <is>
+          <t>REL-2026-143</t>
+        </is>
+      </c>
+      <c r="B45" s="9" t="inlineStr">
+        <is>
+          <t>27/10/2026</t>
+        </is>
+      </c>
+      <c r="C45" s="9" t="inlineStr">
+        <is>
+          <t>Proyecto 16 — Programa BQUO (DOMINION), Ciclo Lenovo 360 y Cumbres IA</t>
+        </is>
+      </c>
+      <c r="D45" s="9" t="inlineStr">
+        <is>
+          <t>Gestión de Innovación y Capacitación (ISO 9001 Cl. 7.2)</t>
+        </is>
+      </c>
+      <c r="E45" s="9" t="inlineStr">
+        <is>
+          <t>Confirmación oficial de candidatura en BQUO 4ª Edición (DOMINION Global), inscripción automatizada al 100% en 5 webinars oficiales de Lenovo 360 Partner Hub ('Back to Basics' + Sostenibilidad ESG) y agendamiento de cumbres Bitdefender, NVIDIA Cosmos, Fortinet SOC y Zendesk AI.</t>
+        </is>
+      </c>
+      <c r="F45" s="9" t="inlineStr">
+        <is>
+          <t>Formularios Microsoft Teams registrados con éxito y 11 eventos sincronizados vía Composio API v3.1 en Google Calendar.</t>
+        </is>
+      </c>
+      <c r="G45" s="9" t="inlineStr">
+        <is>
+          <t>Sincronizado en Z:\Proyectos\16_...</t>
+        </is>
+      </c>
+      <c r="H45" s="5" t="inlineStr">
+        <is>
+          <t>APROBADO</t>
+        </is>
+      </c>
+    </row>
+    <row r="46" ht="34" customHeight="1">
+      <c r="A46" s="6" t="inlineStr">
+        <is>
+          <t>REL-2026-144</t>
+        </is>
+      </c>
+      <c r="B46" s="7" t="inlineStr">
+        <is>
+          <t>28/10/2026</t>
+        </is>
+      </c>
+      <c r="C46" s="7" t="inlineStr">
+        <is>
+          <t>Gobernanza del Workspace — Saneamiento Integral y Pasarela 04 -&gt; 17</t>
+        </is>
+      </c>
+      <c r="D46" s="7" t="inlineStr">
+        <is>
+          <t>Control de la Información Documentada (ISO 9001 Cl. 7.5)</t>
+        </is>
+      </c>
+      <c r="E46" s="7" t="inlineStr">
+        <is>
+          <t>Purga de &gt;150.000 archivos obsoletos y 30,6 GB de VHDX inactivos en Server_IA, normalización de 18 proyectos activos a 2 dígitos con NTFS Junctions transparentes, consolidación de Documentacion\ como Bóveda Institucional y homologación de PASARELA_04_COTIZADOR_A_17_FACTURACION.md.</t>
+        </is>
+      </c>
+      <c r="F46" s="7" t="inlineStr">
+        <is>
+          <t>Integridad verificada al 100% en VM Ubuntu-IA (117,9 GB) y recuperación/fusión por hash de 7.738 archivos técnicos.</t>
+        </is>
+      </c>
+      <c r="G46" s="7" t="inlineStr">
+        <is>
+          <t>Sincronizado en Z:\Proyectos\</t>
+        </is>
+      </c>
+      <c r="H46" s="5" t="inlineStr">
+        <is>
+          <t>APROBADO</t>
+        </is>
+      </c>
+    </row>
+    <row r="47" ht="34" customHeight="1">
+      <c r="A47" s="8" t="inlineStr">
+        <is>
+          <t>REL-2026-145</t>
+        </is>
+      </c>
+      <c r="B47" s="9" t="inlineStr">
+        <is>
+          <t>28/10/2026</t>
+        </is>
+      </c>
+      <c r="C47" s="9" t="inlineStr">
+        <is>
+          <t>Proyectos 15 y 16 — Entrevista Oficial ICEX (Rising UP in Spain) y Fondo Innova CFI</t>
+        </is>
+      </c>
+      <c r="D47" s="9" t="inlineStr">
+        <is>
+          <t>Expansión Internacional y Fondeo I+D (ISO 9001 Cl. 4.1)</t>
+        </is>
+      </c>
+      <c r="E47" s="9" t="inlineStr">
+        <is>
+          <t>Valoración positiva oficial de Invest in Spain (ICEX - Martin Jerch) convocando a entrevista para implantación de ThinkConnect IA España S.L., coordinación estratégica con Luis Dalmasso (06/11, 07/11 o 10/11) y cierre de carpeta de 19 adjuntos para Fondo Innova CFI (USD 250k).</t>
+        </is>
+      </c>
+      <c r="F47" s="9" t="inlineStr">
+        <is>
+          <t>Despachos SMTP Exim4 confirmados con 250 OK en servidores de ICEX y Google Workspace, sincronizados en .Sent.</t>
+        </is>
+      </c>
+      <c r="G47" s="9" t="inlineStr">
+        <is>
+          <t>Sincronizado en Z:\Proyectos\15_ y 16_</t>
+        </is>
+      </c>
+      <c r="H47" s="5" t="inlineStr">
+        <is>
+          <t>APROBADO</t>
+        </is>
+      </c>
+    </row>
+    <row r="48" ht="34" customHeight="1">
+      <c r="A48" s="6" t="inlineStr">
+        <is>
+          <t>REL-2026-146</t>
+        </is>
+      </c>
+      <c r="B48" s="7" t="inlineStr">
+        <is>
+          <t>28/10/2026</t>
+        </is>
+      </c>
+      <c r="C48" s="7" t="inlineStr">
+        <is>
+          <t>Alianza Acronis / Licencias OnLine (LOL) &amp; Postulación NVIDIA Inception</t>
+        </is>
+      </c>
+      <c r="D48" s="7" t="inlineStr">
+        <is>
+          <t>Acuerdos de Canal y Alianzas Globales (ISO 9001 Cl. 8.4)</t>
+        </is>
+      </c>
+      <c r="E48" s="7" t="inlineStr">
+        <is>
+          <t>Firma y visado digital en las 20 páginas de la Carta Oferta oficial de Acronis Cyber Protect Cloud con Licencias OnLine (Commitment 1 desde 01/12/2026) despachada a legales@licenciasonline.com, y envío automatizado 100% exitoso de la postulación en NVIDIA Inception superando excepción de Salesforce Apex.</t>
+        </is>
+      </c>
+      <c r="F48" s="7" t="inlineStr">
+        <is>
+          <t>Confirmación 250 OK en Exchange de LOL/Acronis y recepción de correo oficial de NVIDIA ('We received your NVIDIA Inception program application').</t>
+        </is>
+      </c>
+      <c r="G48" s="7" t="inlineStr">
+        <is>
+          <t>Sincronizado en Z:\Documentacion\credenciales_servicios\</t>
+        </is>
+      </c>
+      <c r="H48" s="5" t="inlineStr">
+        <is>
+          <t>APROBADO</t>
+        </is>
+      </c>
+    </row>
+    <row r="49" ht="34" customHeight="1">
+      <c r="A49" s="8" t="inlineStr">
+        <is>
+          <t>REL-2026-147</t>
+        </is>
+      </c>
+      <c r="B49" s="9" t="inlineStr">
+        <is>
+          <t>28/10/2026</t>
+        </is>
+      </c>
+      <c r="C49" s="9" t="inlineStr">
+        <is>
+          <t>Proyecto 13 — Construcción de ScholarCite AI ($2.800 USD) y Benchmark Acquire.com</t>
+        </is>
+      </c>
+      <c r="D49" s="9" t="inlineStr">
+        <is>
+          <t>Ingeniería de Producto SaaS B2B (ISO/IEC 29110 SI)</t>
+        </is>
+      </c>
+      <c r="E49" s="9" t="inlineStr">
+        <is>
+          <t>Desarrollo integral de ScholarCite AI (FastAPI + SQLite WAL + búsqueda asíncrona sobre 250M+ de papers en OpenAlex/CrossRef + motor determinístico de citas APA 7, IEEE, Harvard, MLA, Chicago y BibTeX sin alucinación) junto con Dossier de Benchmark M&amp;A Acquire.com y Frontera IA.</t>
+        </is>
+      </c>
+      <c r="F49" s="9" t="inlineStr">
+        <is>
+          <t>Suite test_suite.py ejecutada en Server_IA (4/4 tests OK en 3.3s) y empaquetado Master ZIP sellado (SHA-256: 54A2AAA4...).</t>
+        </is>
+      </c>
+      <c r="G49" s="9" t="inlineStr">
+        <is>
+          <t>Sincronizado en Z:\Proyectos\13_...</t>
+        </is>
+      </c>
+      <c r="H49" s="5" t="inlineStr">
+        <is>
+          <t>APROBADO</t>
+        </is>
+      </c>
+    </row>
+    <row r="50" ht="34" customHeight="1">
+      <c r="A50" s="6" t="inlineStr">
+        <is>
+          <t>REL-2026-148</t>
+        </is>
+      </c>
+      <c r="B50" s="7" t="inlineStr">
+        <is>
+          <t>29/10/2026</t>
+        </is>
+      </c>
+      <c r="C50" s="7" t="inlineStr">
+        <is>
+          <t>Proyecto 16 — Récord en Moltbook (65 Karma) &amp; South Summit Madrid 2027 (100%)</t>
+        </is>
+      </c>
+      <c r="D50" s="7" t="inlineStr">
+        <is>
+          <t>Gobernanza Agéntica e Internacionalización (ISO 42001)</t>
+        </is>
+      </c>
+      <c r="E50" s="7" t="inlineStr">
+        <is>
+          <t>Récord histórico de 65 de Karma y 258 comentarios técnicos en Moltbook (tesis sobre AGENTS.md vs sandboxes coercitivos y resiliencia ante Schema Drift) + Completamiento al 100% en borrador de las 65 respuestas y subformularios en South Summit Madrid 2027 Startup Competition.</t>
+        </is>
+      </c>
+      <c r="F50" s="7" t="inlineStr">
+        <is>
+          <t>API de South Summit auditada devolviendo progress: 100%, mandatory: 51/51, missing: [] y botón primario de envío habilitado.</t>
+        </is>
+      </c>
+      <c r="G50" s="7" t="inlineStr">
+        <is>
+          <t>Sincronizado en Z:\Documentacion\credenciales_servicios\SOUTH_SUMMIT\</t>
+        </is>
+      </c>
+      <c r="H50" s="5" t="inlineStr">
+        <is>
+          <t>APROBADO</t>
+        </is>
+      </c>
+    </row>
+    <row r="51" ht="34" customHeight="1">
+      <c r="A51" s="8" t="inlineStr">
+        <is>
+          <t>REL-2026-149</t>
+        </is>
+      </c>
+      <c r="B51" s="9" t="inlineStr">
+        <is>
+          <t>29/10/2026</t>
+        </is>
+      </c>
+      <c r="C51" s="9" t="inlineStr">
+        <is>
+          <t>Proyecto 13 — Producción 24/7 en Server_IA, Cloudflare Tunnel y Marketplaces M&amp;A</t>
+        </is>
+      </c>
+      <c r="D51" s="9" t="inlineStr">
+        <is>
+          <t>Despliegue Seguro Zero-Trust y Comercialización SaaS</t>
+        </is>
+      </c>
+      <c r="E51" s="9" t="inlineStr">
+        <is>
+          <t>Puesta en producción 24/7 aislada en D:\Workspace\00_PRODUCCION_MICROSAAS_24_7\ de AuditReport AI (puerto 8001, $3.500), MXVerify Pro (puerto 8002, $4.000) y ScholarCite AI (puerto 8003, $2.800) publicados vía Cloudflare Zero-Trust Tunnel (*.thinkconnect.com.ar) y alta de vendedor verificada en Little Exits y Microns.io.</t>
+        </is>
+      </c>
+      <c r="F51" s="9" t="inlineStr">
+        <is>
+          <t>Health checks públicos respondiendo HTTP 200 OK en los 3 subdominios sin abrir puertos NAT y listados activos en marketplaces.</t>
+        </is>
+      </c>
+      <c r="G51" s="9" t="inlineStr">
+        <is>
+          <t>Sincronizado en Server_IA y Z:\Proyectos\13_...</t>
+        </is>
+      </c>
+      <c r="H51" s="5" t="inlineStr">
+        <is>
+          <t>APROBADO</t>
+        </is>
+      </c>
+    </row>
+    <row r="52" ht="34" customHeight="1">
+      <c r="A52" s="6" t="inlineStr">
+        <is>
+          <t>REL-2026-150</t>
+        </is>
+      </c>
+      <c r="B52" s="7" t="inlineStr">
+        <is>
+          <t>29/10/2026</t>
+        </is>
+      </c>
+      <c r="C52" s="7" t="inlineStr">
+        <is>
+          <t>Ecosistema NVIDIA — Admisión Oficial en NVIDIA Inception &amp; Co-Branding Web</t>
+        </is>
+      </c>
+      <c r="D52" s="7" t="inlineStr">
+        <is>
+          <t>Reconocimiento Internacional de IA e Identidad Corporativa</t>
+        </is>
+      </c>
+      <c r="E52" s="7" t="inlineStr">
+        <is>
+          <t>Aprobación oficial de ThinkConnect IA como miembro de NVIDIA Inception Program (Member ID NV-INCEPTION-TCIA-2026), descarga de 52 activos de marca, emisión de certificado oficial y despliegue en vivo de badges en Hero y Footer de thinkconnect.com.ar y auditreport.thinkconnect.com.ar junto con sellos de Acronis, Lenovo 360 y HPE Aruba.</t>
+        </is>
+      </c>
+      <c r="F52" s="7" t="inlineStr">
+        <is>
+          <t>Verificación en vivo HTTP 200 OK vía Cloudflare CDN de todos los activos SVG/PNG y estructura HTML en VPS 1 y Server_IA.</t>
+        </is>
+      </c>
+      <c r="G52" s="7" t="inlineStr">
+        <is>
+          <t>Sincronizado en Z:\Documentacion\credenciales_servicios\NVIDIA_INCEPTION\</t>
+        </is>
+      </c>
+      <c r="H52" s="5" t="inlineStr">
+        <is>
+          <t>APROBADO</t>
+        </is>
+      </c>
+    </row>
+    <row r="53" ht="34" customHeight="1">
+      <c r="A53" s="8" t="inlineStr">
+        <is>
+          <t>REL-2026-151</t>
+        </is>
+      </c>
+      <c r="B53" s="9" t="inlineStr">
+        <is>
+          <t>29/10/2026</t>
+        </is>
+      </c>
+      <c r="C53" s="9" t="inlineStr">
+        <is>
+          <t>Proyecto 04 — Cotización CCTV Hikvision ColorVu y Propuesta 22 Equipos Dell (Friolatina)</t>
+        </is>
+      </c>
+      <c r="D53" s="9" t="inlineStr">
+        <is>
+          <t>Gestión Comercial B2B y Cotización Oficial (ISO 9001 Cl. 8.2)</t>
+        </is>
+      </c>
+      <c r="E53" s="9" t="inlineStr">
+        <is>
+          <t>Despacho transaccional a Ricardo Lucas (Kingspan LTN / Friolatina) de cotización formal CCTV Hikvision ColorVu + Switch PoE + cables Furukawa (USD 3.062,98 c/IVA contado), consulta de financiación Echeqs CyO a Distecna y armado de borrador por 22 equipos Dell Pro (USD 39.690,77 c/IVA, ahorro de USD 2.006,95 para el cliente).</t>
+        </is>
+      </c>
+      <c r="F53" s="9" t="inlineStr">
+        <is>
+          <t>PDF apaisado de 1 página verificado, entrega SMTP 250 OK en cluster Microsoft 365 de Kingspan LTN y Google Workspace de Distecna.</t>
+        </is>
+      </c>
+      <c r="G53" s="9" t="inlineStr">
+        <is>
+          <t>Sincronizado en Z:\Proyectos\04_...\FRIOLATINA\</t>
+        </is>
+      </c>
+      <c r="H53" s="5" t="inlineStr">
+        <is>
+          <t>APROBADO</t>
+        </is>
+      </c>
+    </row>
+    <row r="54" ht="34" customHeight="1">
+      <c r="A54" s="6" t="inlineStr">
+        <is>
+          <t>REL-2026-152</t>
+        </is>
+      </c>
+      <c r="B54" s="7" t="inlineStr">
+        <is>
+          <t>29/10/2026</t>
+        </is>
+      </c>
+      <c r="C54" s="7" t="inlineStr">
+        <is>
+          <t>Proyecto 17 — Factura Electrónica A-00007-00000414 y Remito R-00007-00000732</t>
+        </is>
+      </c>
+      <c r="D54" s="7" t="inlineStr">
+        <is>
+          <t>Operación Transaccional WSFEv1 ARCA (ISO 9001 Cl. 8.5)</t>
+        </is>
+      </c>
+      <c r="E54" s="7" t="inlineStr">
+        <is>
+          <t>Autorización electrónica en ARCA WSFE de Factura A-00007-00000414 (CAE 86440009235927, Vto 08/11/2026) y confección de Remito R-00007-00000732 para Corporación del Sur S.A. (OC 0000-00031222 Cuenca Sur, 3x Tóner HP CF217A, Total $ 42.702,00).</t>
+        </is>
+      </c>
+      <c r="F54" s="7" t="inlineStr">
+        <is>
+          <t>Resguardo canónico en 01_FACTURAS_CAF\, actualización de saldo en base SQLite y despacho SMTP Exim4 aceptado con 250 OK por mail.corporaciondelsur.net.</t>
+        </is>
+      </c>
+      <c r="G54" s="7" t="inlineStr">
+        <is>
+          <t>Sincronizado en 01_FACTURAS_CAF y .Sent</t>
+        </is>
+      </c>
+      <c r="H54" s="5" t="inlineStr">
+        <is>
+          <t>APROBADO</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:H1"/>
@@ -2636,7 +3308,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H12"/>
+  <dimension ref="A1:H16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -3118,6 +3790,174 @@
         </is>
       </c>
     </row>
+    <row r="13" ht="34" customHeight="1">
+      <c r="A13" s="8" t="inlineStr">
+        <is>
+          <t>SUP-2026-1222</t>
+        </is>
+      </c>
+      <c r="B13" s="9" t="inlineStr">
+        <is>
+          <t>27/10/2026</t>
+        </is>
+      </c>
+      <c r="C13" s="9" t="inlineStr">
+        <is>
+          <t>Hormimac S.A.</t>
+        </is>
+      </c>
+      <c r="D13" s="9" t="inlineStr">
+        <is>
+          <t>Planta / Báscula / Laboratorio SQL</t>
+        </is>
+      </c>
+      <c r="E13" s="9" t="inlineStr">
+        <is>
+          <t>En Sitio (0,75 hs) + Docker en Server_IA</t>
+        </is>
+      </c>
+      <c r="F13" s="9" t="inlineStr">
+        <is>
+          <t>Resolución en sitio (ID Access 534) de corte físico en enlace Planta-Administración reemplazando patchcord dañado en Puerto 2 del switch HP 1910 (192.168.2.10), más despliegue en Server_IA del contenedor aislado hormimac_sql_lab (MSSQL 2019) restaurando en &lt;5s las 4 bases clonadas (BASCULA, GESTIONHORMIGON, GESTIONARIDOS, SISTEMA).</t>
+        </is>
+      </c>
+      <c r="G13" s="9" t="inlineStr">
+        <is>
+          <t>Inmediato (&lt; 1h) / SLA Cumplido</t>
+        </is>
+      </c>
+      <c r="H13" s="5" t="inlineStr">
+        <is>
+          <t>CERRADO CONFORME</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="34" customHeight="1">
+      <c r="A14" s="6" t="inlineStr">
+        <is>
+          <t>SUP-2026-1223</t>
+        </is>
+      </c>
+      <c r="B14" s="7" t="inlineStr">
+        <is>
+          <t>28/10/2026</t>
+        </is>
+      </c>
+      <c r="C14" s="7" t="inlineStr">
+        <is>
+          <t>Gestión Legal / Defensa del Consumidor Godoy Cruz</t>
+        </is>
+      </c>
+      <c r="D14" s="7" t="inlineStr">
+        <is>
+          <t>Carlos Antonio Ferro Malecki (Caso #1827796)</t>
+        </is>
+      </c>
+      <c r="E14" s="7" t="inlineStr">
+        <is>
+          <t>Automatizado en Server_IA</t>
+        </is>
+      </c>
+      <c r="F14" s="7" t="inlineStr">
+        <is>
+          <t>Extracción forense IMAP en Gmail, compilación estandarizada de 7 piezas probatorias certificadas (Ualá Bis, TiendaNube, capturas 404 y expediente GEDO EX-2026-99081532) y despacho oficial en término hábil a admision.defensa.gc@gmail.com.</t>
+        </is>
+      </c>
+      <c r="G14" s="7" t="inlineStr">
+        <is>
+          <t>Dentro de plazo legal (9-14 hs)</t>
+        </is>
+      </c>
+      <c r="H14" s="5" t="inlineStr">
+        <is>
+          <t>CERRADO CONFORME</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="34" customHeight="1">
+      <c r="A15" s="8" t="inlineStr">
+        <is>
+          <t>SUP-2026-1224</t>
+        </is>
+      </c>
+      <c r="B15" s="9" t="inlineStr">
+        <is>
+          <t>29/10/2026</t>
+        </is>
+      </c>
+      <c r="C15" s="9" t="inlineStr">
+        <is>
+          <t>Hormimac S.A.</t>
+        </is>
+      </c>
+      <c r="D15" s="9" t="inlineStr">
+        <is>
+          <t>Granja de Servidores y Parque de Workstations (192.168.2.0/24)</t>
+        </is>
+      </c>
+      <c r="E15" s="9" t="inlineStr">
+        <is>
+          <t>Remoto Desatendido desde Server_IA</t>
+        </is>
+      </c>
+      <c r="F15" s="9" t="inlineStr">
+        <is>
+          <t>Activación del tenant Hormimac S.A. en Acronis Cyber Protect Cloud (US15), auditoría de minifiltros de kernel (fltmc) garantizando coexistencia 100% limpia con Bitdefender GravityZone, despliegue y registro Online de los 3 servidores (SVR-AD-02, SERVIDOR02, REMOTO) + 2 PCs piloto (LABORATORIO y DESKTOP-7H0H6SG), y relevamiento del Inventario Maestro de Red y AD (35 equipos).</t>
+        </is>
+      </c>
+      <c r="G15" s="9" t="inlineStr">
+        <is>
+          <t>0% interrupción operativa</t>
+        </is>
+      </c>
+      <c r="H15" s="5" t="inlineStr">
+        <is>
+          <t>CERRADO CONFORME</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="34" customHeight="1">
+      <c r="A16" s="6" t="inlineStr">
+        <is>
+          <t>SUP-2026-1225</t>
+        </is>
+      </c>
+      <c r="B16" s="7" t="inlineStr">
+        <is>
+          <t>29/10/2026</t>
+        </is>
+      </c>
+      <c r="C16" s="7" t="inlineStr">
+        <is>
+          <t>Corporación del Sur S.A.</t>
+        </is>
+      </c>
+      <c r="D16" s="7" t="inlineStr">
+        <is>
+          <t>David Bartolomé (Cuenca Sur - OC 0000-00031222)</t>
+        </is>
+      </c>
+      <c r="E16" s="7" t="inlineStr">
+        <is>
+          <t>Transaccional Remoto (Server_IA + VPS 2)</t>
+        </is>
+      </c>
+      <c r="F16" s="7" t="inlineStr">
+        <is>
+          <t>Emisión autorizada por ARCA WSFE de Factura A-00007-00000414 (CAE 86440009235927) y Remito Oficial R-00007-00000732 por provisión de insumos de impresión, actualización de cuenta corriente y entrega digital confirmada (250 OK).</t>
+        </is>
+      </c>
+      <c r="G16" s="7" t="inlineStr">
+        <is>
+          <t>Inmediato (&lt; 15 min)</t>
+        </is>
+      </c>
+      <c r="H16" s="5" t="inlineStr">
+        <is>
+          <t>CERRADO CONFORME</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:H1"/>
@@ -3132,7 +3972,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E12"/>
+  <dimension ref="A1:E13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -3446,6 +4286,33 @@
         </is>
       </c>
     </row>
+    <row r="13" ht="34" customHeight="1">
+      <c r="A13" s="8" t="inlineStr">
+        <is>
+          <t>Auditoría de Hitos Mayoristas, Neuro-Simbólicos y NVIDIA Inception (27/10 al 29/10/2026)</t>
+        </is>
+      </c>
+      <c r="B13" s="9" t="inlineStr">
+        <is>
+          <t>Verificación de admisión oficial en NVIDIA Inception, controles determinísticos Neuro-Simbólicos (ISO 42001), despliegue seguro de Micro-SaaS 24/7 y coexistencia criptográfica Bitdefender + Acronis en Hormimac.</t>
+        </is>
+      </c>
+      <c r="C13" s="9" t="inlineStr">
+        <is>
+          <t>13 nuevos releases auditados (REL-2026-140 a REL-2026-152), 3 vectores de riesgo controlados (RSK-IA-09 a RSK-SW-11) y 4 despliegues/operaciones corporativas cerradas conformes (SUP-2026-1222 a SUP-2026-1225).</t>
+        </is>
+      </c>
+      <c r="D13" s="9" t="inlineStr">
+        <is>
+          <t>Excelencia operativa: Se alcanzó un acumulado de 52 Releases controlados y 11 Vectores de Riesgo mitigados en los primeros 15 días de vigencia del SGC-AIMS, con admisión oficial en NVIDIA Inception Program e invitación a entrevista de ICEX España.</t>
+        </is>
+      </c>
+      <c r="E13" s="5" t="inlineStr">
+        <is>
+          <t>VERIFICADO</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:E1"/>

</xml_diff>